<commit_message>
Ingesta diaria 2026-09-22 09:28
</commit_message>
<xml_diff>
--- a/data/Campos_actual.xlsx
+++ b/data/Campos_actual.xlsx
@@ -691,7 +691,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>1</v>
@@ -811,7 +815,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>1</v>
@@ -1018,7 +1026,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1047,7 +1055,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>1</v>
@@ -1070,7 +1082,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1096,7 +1108,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1122,10 +1134,14 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>En proceso</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>1</v>
@@ -1268,7 +1284,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1414,7 +1430,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1448,7 +1464,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -1534,7 +1550,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -1802,7 +1818,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -1948,7 +1964,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2089,7 +2105,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
         <v>1</v>
@@ -2224,7 +2244,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2305,7 +2325,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
         <v>1</v>
@@ -2432,7 +2456,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -2802,7 +2826,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -2828,7 +2852,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -2958,7 +2982,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3138,7 +3162,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -3271,7 +3295,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="n">
         <v>1</v>
@@ -3323,7 +3351,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="n">
         <v>1</v>
@@ -3372,7 +3404,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -3710,7 +3742,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -3970,7 +4002,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -4516,7 +4548,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
@@ -4545,7 +4577,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G149" t="inlineStr"/>
       <c r="H149" t="n">
         <v>1</v>
@@ -4568,7 +4604,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -4602,7 +4638,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F151" t="inlineStr"/>
@@ -4665,7 +4701,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G153" t="inlineStr"/>
       <c r="H153" t="n">
         <v>1</v>
@@ -4725,7 +4765,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G155" t="inlineStr"/>
       <c r="H155" t="n">
         <v>1</v>
@@ -4881,7 +4925,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr"/>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G161" t="inlineStr"/>
       <c r="H161" t="n">
         <v>1</v>
@@ -4967,7 +5015,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="n">
         <v>1</v>
@@ -4990,7 +5042,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -5019,7 +5071,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G166" t="inlineStr"/>
       <c r="H166" t="n">
         <v>1</v>
@@ -5045,7 +5101,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr"/>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G167" t="inlineStr"/>
       <c r="H167" t="n">
         <v>1</v>
@@ -5071,7 +5131,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G168" t="inlineStr"/>
       <c r="H168" t="n">
         <v>1</v>
@@ -5120,7 +5184,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
@@ -5146,7 +5210,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -5180,7 +5244,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F172" t="inlineStr"/>
@@ -5295,7 +5359,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F176" t="inlineStr"/>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="n">
         <v>1</v>
@@ -5347,7 +5415,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="n">
         <v>1</v>
@@ -5508,7 +5580,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -5638,7 +5710,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
@@ -5758,7 +5830,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F193" t="inlineStr"/>
@@ -5784,7 +5856,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -5839,7 +5911,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr"/>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="n">
         <v>1</v>
@@ -5862,7 +5938,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
@@ -5940,10 +6016,14 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F200" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="n">
         <v>1</v>
@@ -5969,7 +6049,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr"/>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="n">
         <v>1</v>
@@ -6115,7 +6199,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="n">
         <v>1</v>
@@ -6227,7 +6315,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="n">
         <v>1</v>
@@ -6284,7 +6376,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F212" t="inlineStr"/>
@@ -6756,7 +6848,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -6824,7 +6916,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -6947,7 +7039,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr"/>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G234" t="inlineStr"/>
       <c r="H234" t="n">
         <v>1</v>
@@ -7004,7 +7100,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
@@ -7106,7 +7202,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -7271,7 +7367,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr"/>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G244" t="inlineStr"/>
       <c r="H244" t="n">
         <v>1</v>
@@ -7365,7 +7465,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G247" t="inlineStr"/>
       <c r="H247" t="n">
         <v>1</v>
@@ -7425,7 +7529,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G249" t="inlineStr"/>
       <c r="H249" t="n">
         <v>1</v>
@@ -7553,7 +7661,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F253" t="inlineStr"/>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G253" t="inlineStr"/>
       <c r="H253" t="n">
         <v>1</v>
@@ -7715,7 +7827,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F258" t="inlineStr"/>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G258" t="inlineStr"/>
       <c r="H258" t="n">
         <v>1</v>
@@ -7741,7 +7857,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr"/>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G259" t="inlineStr"/>
       <c r="H259" t="n">
         <v>1</v>
@@ -7790,7 +7910,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -7913,7 +8033,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F265" t="inlineStr"/>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G265" t="inlineStr"/>
       <c r="H265" t="n">
         <v>1</v>
@@ -8066,7 +8190,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F271" t="inlineStr"/>
@@ -8298,7 +8422,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F279" t="inlineStr"/>
@@ -8561,7 +8685,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr"/>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G289" t="inlineStr"/>
       <c r="H289" t="n">
         <v>1</v>
@@ -8636,7 +8764,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F292" t="inlineStr"/>
@@ -8665,7 +8793,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F293" t="inlineStr"/>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G293" t="inlineStr"/>
       <c r="H293" t="n">
         <v>1</v>
@@ -8714,7 +8846,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F295" t="inlineStr"/>
@@ -8766,7 +8898,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F297" t="inlineStr"/>
@@ -8844,7 +8976,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F300" t="inlineStr"/>
@@ -8870,7 +9002,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F301" t="inlineStr"/>
@@ -9026,7 +9158,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F307" t="inlineStr"/>
@@ -9133,7 +9265,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F311" t="inlineStr"/>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G311" t="inlineStr"/>
       <c r="H311" t="n">
         <v>1</v>
@@ -9185,7 +9321,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F313" t="inlineStr"/>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G313" t="inlineStr"/>
       <c r="H313" t="n">
         <v>1</v>
@@ -9390,7 +9530,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F321" t="inlineStr"/>
@@ -9445,7 +9585,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr"/>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G323" t="inlineStr"/>
       <c r="H323" t="n">
         <v>1</v>
@@ -9471,7 +9615,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F324" t="inlineStr"/>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G324" t="inlineStr"/>
       <c r="H324" t="n">
         <v>1</v>
@@ -9497,7 +9645,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F325" t="inlineStr"/>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G325" t="inlineStr"/>
       <c r="H325" t="n">
         <v>1</v>
@@ -9520,7 +9672,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F326" t="inlineStr"/>
@@ -9546,7 +9698,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F327" t="inlineStr"/>
@@ -9754,7 +9906,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F335" t="inlineStr"/>
@@ -9806,7 +9958,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F337" t="inlineStr"/>
@@ -10004,7 +10156,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F344" t="inlineStr"/>
@@ -10030,7 +10182,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F345" t="inlineStr"/>
@@ -10220,7 +10372,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F352" t="inlineStr"/>
@@ -10246,10 +10398,14 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F353" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G353" t="inlineStr"/>
       <c r="H353" t="n">
         <v>1</v>
@@ -10272,10 +10428,14 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F354" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G354" t="inlineStr"/>
       <c r="H354" t="n">
         <v>1</v>
@@ -10350,7 +10510,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F357" t="inlineStr"/>
@@ -10696,7 +10856,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F370" t="inlineStr"/>
@@ -10800,10 +10960,14 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F374" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G374" t="inlineStr"/>
       <c r="H374" t="n">
         <v>1</v>
@@ -10852,7 +11016,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F376" t="inlineStr"/>
@@ -10956,10 +11120,14 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F380" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G380" t="inlineStr"/>
       <c r="H380" t="n">
         <v>1</v>
@@ -11570,7 +11738,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F403" t="inlineStr"/>
@@ -11596,7 +11764,7 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F404" t="inlineStr"/>
@@ -11968,7 +12136,7 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F418" t="inlineStr"/>
@@ -12176,7 +12344,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F426" t="inlineStr"/>
@@ -12228,7 +12396,7 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F428" t="inlineStr"/>
@@ -12306,7 +12474,7 @@
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F431" t="inlineStr"/>
@@ -12514,7 +12682,7 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F439" t="inlineStr"/>
@@ -12722,7 +12890,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F447" t="inlineStr"/>
@@ -12837,7 +13005,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F451" t="inlineStr"/>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G451" t="inlineStr"/>
       <c r="H451" t="n">
         <v>1</v>
@@ -12863,7 +13035,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F452" t="inlineStr"/>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G452" t="inlineStr"/>
       <c r="H452" t="n">
         <v>1</v>
@@ -12889,7 +13065,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F453" t="inlineStr"/>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G453" t="inlineStr"/>
       <c r="H453" t="n">
         <v>1</v>
@@ -12949,7 +13129,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F455" t="inlineStr"/>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G455" t="inlineStr"/>
       <c r="H455" t="n">
         <v>1</v>
@@ -13001,7 +13185,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F457" t="inlineStr"/>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G457" t="inlineStr"/>
       <c r="H457" t="n">
         <v>1</v>
@@ -13079,7 +13267,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F460" t="inlineStr"/>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G460" t="inlineStr"/>
       <c r="H460" t="n">
         <v>1</v>
@@ -13206,7 +13398,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F465" t="inlineStr"/>
@@ -13310,7 +13502,7 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F469" t="inlineStr"/>
@@ -13336,7 +13528,7 @@
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F470" t="inlineStr"/>
@@ -13648,7 +13840,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F482" t="inlineStr"/>
@@ -13807,7 +13999,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F488" t="inlineStr"/>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G488" t="inlineStr"/>
       <c r="H488" t="n">
         <v>1</v>
@@ -13830,7 +14026,7 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F489" t="inlineStr">
@@ -13935,7 +14131,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F492" t="inlineStr"/>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G492" t="inlineStr"/>
       <c r="H492" t="n">
         <v>2</v>
@@ -14120,7 +14320,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F498" t="inlineStr">
@@ -14157,7 +14357,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F499" t="inlineStr"/>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G499" t="inlineStr"/>
       <c r="H499" t="n">
         <v>1</v>
@@ -14287,7 +14491,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F504" t="inlineStr"/>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G504" t="inlineStr"/>
       <c r="H504" t="n">
         <v>1</v>
@@ -14336,7 +14544,7 @@
       </c>
       <c r="E506" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F506" t="inlineStr">
@@ -14485,7 +14693,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F511" t="inlineStr"/>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G511" t="inlineStr"/>
       <c r="H511" t="n">
         <v>1</v>
@@ -14589,7 +14801,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F515" t="inlineStr"/>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G515" t="inlineStr"/>
       <c r="H515" t="n">
         <v>1</v>
@@ -14849,7 +15065,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F525" t="inlineStr"/>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G525" t="inlineStr"/>
       <c r="H525" t="n">
         <v>1</v>
@@ -15029,7 +15249,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F531" t="inlineStr"/>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G531" t="inlineStr"/>
       <c r="H531" t="n">
         <v>1</v>
@@ -15107,7 +15331,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F534" t="inlineStr"/>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G534" t="inlineStr"/>
       <c r="H534" t="n">
         <v>1</v>
@@ -15364,7 +15592,7 @@
       </c>
       <c r="E544" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F544" t="inlineStr"/>
@@ -15416,7 +15644,7 @@
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F546" t="inlineStr"/>
@@ -15624,7 +15852,7 @@
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F554" t="inlineStr"/>
@@ -15702,7 +15930,7 @@
       </c>
       <c r="E557" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F557" t="inlineStr"/>
@@ -15835,7 +16063,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F562" t="inlineStr"/>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G562" t="inlineStr"/>
       <c r="H562" t="n">
         <v>1</v>
@@ -16274,7 +16506,7 @@
       </c>
       <c r="E579" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F579" t="inlineStr"/>
@@ -16300,7 +16532,7 @@
       </c>
       <c r="E580" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F580" t="inlineStr"/>
@@ -17984,7 +18216,7 @@
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F642" t="inlineStr"/>
@@ -18036,7 +18268,7 @@
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F644" t="inlineStr"/>
@@ -18096,7 +18328,7 @@
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F646" t="inlineStr"/>
@@ -18125,7 +18357,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F647" t="inlineStr"/>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G647" t="inlineStr"/>
       <c r="H647" t="n">
         <v>1</v>
@@ -18260,7 +18496,7 @@
       </c>
       <c r="E652" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F652" t="inlineStr"/>
@@ -18289,7 +18525,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F653" t="inlineStr"/>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G653" t="inlineStr"/>
       <c r="H653" t="n">
         <v>1</v>
@@ -18338,7 +18578,7 @@
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F655" t="inlineStr"/>
@@ -18401,7 +18641,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F657" t="inlineStr"/>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G657" t="inlineStr"/>
       <c r="H657" t="n">
         <v>1</v>
@@ -18427,7 +18671,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F658" t="inlineStr"/>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G658" t="inlineStr"/>
       <c r="H658" t="n">
         <v>1</v>
@@ -18453,7 +18701,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F659" t="inlineStr"/>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G659" t="inlineStr"/>
       <c r="H659" t="n">
         <v>1</v>
@@ -18539,7 +18791,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F662" t="inlineStr"/>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G662" t="inlineStr"/>
       <c r="H662" t="n">
         <v>1</v>
@@ -18599,7 +18855,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F664" t="inlineStr"/>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G664" t="inlineStr"/>
       <c r="H664" t="n">
         <v>1</v>
@@ -18651,7 +18911,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F666" t="inlineStr"/>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G666" t="inlineStr"/>
       <c r="H666" t="n">
         <v>1</v>
@@ -18703,7 +18967,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F668" t="inlineStr"/>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G668" t="inlineStr"/>
       <c r="H668" t="n">
         <v>1</v>
@@ -18755,7 +19023,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F670" t="inlineStr"/>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G670" t="inlineStr"/>
       <c r="H670" t="n">
         <v>1</v>
@@ -18937,7 +19209,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F677" t="inlineStr"/>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G677" t="inlineStr"/>
       <c r="H677" t="n">
         <v>1</v>
@@ -18989,7 +19265,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F679" t="inlineStr"/>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G679" t="inlineStr"/>
       <c r="H679" t="n">
         <v>1</v>
@@ -19015,7 +19295,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F680" t="inlineStr"/>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G680" t="inlineStr"/>
       <c r="H680" t="n">
         <v>1</v>
@@ -19090,7 +19374,7 @@
       </c>
       <c r="E683" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F683" t="inlineStr"/>
@@ -19171,7 +19455,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F686" t="inlineStr"/>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G686" t="inlineStr"/>
       <c r="H686" t="n">
         <v>1</v>
@@ -19194,7 +19482,7 @@
       </c>
       <c r="E687" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F687" t="inlineStr"/>
@@ -19324,7 +19612,7 @@
       </c>
       <c r="E692" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F692" t="inlineStr"/>
@@ -19457,7 +19745,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F697" t="inlineStr"/>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G697" t="inlineStr"/>
       <c r="H697" t="n">
         <v>1</v>
@@ -19613,7 +19905,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F703" t="inlineStr"/>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G703" t="inlineStr"/>
       <c r="H703" t="n">
         <v>1</v>
@@ -19759,7 +20055,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F708" t="inlineStr"/>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G708" t="inlineStr"/>
       <c r="H708" t="n">
         <v>1</v>
@@ -19816,7 +20116,7 @@
       </c>
       <c r="E710" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F710" t="inlineStr">
@@ -19853,7 +20153,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F711" t="inlineStr"/>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G711" t="inlineStr"/>
       <c r="H711" t="n">
         <v>1</v>
@@ -19910,7 +20214,7 @@
       </c>
       <c r="E713" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F713" t="inlineStr"/>
@@ -20085,7 +20389,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F719" t="inlineStr"/>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G719" t="inlineStr"/>
       <c r="H719" t="n">
         <v>1</v>
@@ -20223,7 +20531,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F724" t="inlineStr"/>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G724" t="inlineStr"/>
       <c r="H724" t="n">
         <v>1</v>
@@ -20249,7 +20561,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F725" t="inlineStr"/>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G725" t="inlineStr"/>
       <c r="H725" t="n">
         <v>1</v>
@@ -20473,7 +20789,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F733" t="inlineStr"/>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G733" t="inlineStr"/>
       <c r="H733" t="n">
         <v>1</v>
@@ -20814,7 +21134,7 @@
       </c>
       <c r="E745" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F745" t="inlineStr">
@@ -20848,7 +21168,7 @@
       </c>
       <c r="E746" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F746" t="inlineStr">
@@ -21067,7 +21387,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F754" t="inlineStr"/>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G754" t="inlineStr"/>
       <c r="H754" t="n">
         <v>1</v>
@@ -21093,7 +21417,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F755" t="inlineStr"/>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G755" t="inlineStr"/>
       <c r="H755" t="n">
         <v>1</v>
@@ -21119,7 +21447,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F756" t="inlineStr"/>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G756" t="inlineStr"/>
       <c r="H756" t="n">
         <v>1</v>
@@ -21145,7 +21477,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F757" t="inlineStr"/>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G757" t="inlineStr"/>
       <c r="H757" t="n">
         <v>1</v>
@@ -21197,7 +21533,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F759" t="inlineStr"/>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G759" t="inlineStr"/>
       <c r="H759" t="n">
         <v>1</v>
@@ -21223,7 +21563,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F760" t="inlineStr"/>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G760" t="inlineStr"/>
       <c r="H760" t="n">
         <v>1</v>
@@ -21249,7 +21593,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F761" t="inlineStr"/>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G761" t="inlineStr"/>
       <c r="H761" t="n">
         <v>1</v>
@@ -21332,7 +21680,7 @@
       </c>
       <c r="E764" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F764" t="inlineStr"/>
@@ -21384,7 +21732,7 @@
       </c>
       <c r="E766" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F766" t="inlineStr"/>
@@ -21444,7 +21792,7 @@
       </c>
       <c r="E768" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F768" t="inlineStr">
@@ -21478,7 +21826,7 @@
       </c>
       <c r="E769" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F769" t="inlineStr">
@@ -21830,7 +22178,7 @@
       </c>
       <c r="E781" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F781" t="inlineStr"/>
@@ -22090,7 +22438,7 @@
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F791" t="inlineStr"/>
@@ -22116,7 +22464,7 @@
       </c>
       <c r="E792" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F792" t="inlineStr"/>
@@ -22739,7 +23087,11 @@
           <t>En proceso</t>
         </is>
       </c>
-      <c r="F816" t="inlineStr"/>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G816" t="inlineStr"/>
       <c r="H816" t="inlineStr"/>
     </row>
@@ -22763,7 +23115,11 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F817" t="inlineStr"/>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G817" t="inlineStr"/>
       <c r="H817" t="inlineStr"/>
     </row>
@@ -22787,7 +23143,11 @@
           <t>En proceso</t>
         </is>
       </c>
-      <c r="F818" t="inlineStr"/>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G818" t="inlineStr"/>
       <c r="H818" t="inlineStr"/>
     </row>
@@ -22968,7 +23328,7 @@
       </c>
       <c r="E825" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F825" t="inlineStr">
@@ -23335,7 +23695,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Biométrico se encuentra como siniestro hurto pero en realidad esta en la oficina en uso operativo, se encuentra como "NO" facturable</t>
+          <t>Biométrico se encuentra como siniestro hurto pero en realidad esta en la oficina en uso operativo, se encuentra como "NO" facturable, Ssi no se aprueba se debe recoger</t>
         </is>
       </c>
     </row>
@@ -23509,47 +23869,33 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1484</v>
-      </c>
-      <c r="B10" t="n">
-        <v>1484</v>
-      </c>
+        <v>1573</v>
+      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" s="2" t="n">
         <v>46269</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>H_4d9160c1baed</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>VALDIVIA</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Asignado</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
+          <t>H_86189370e5df</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>VALDIVIA</t>
+          <t>SANTA ROSA DE VITERBO</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Antioquia</t>
+          <t>Boyacá</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>INSARED</t>
+          <t>GESTIONATECH</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -23559,29 +23905,43 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Biometrico no esta siendo utilizado, por favor enviar area logistica para la recogida</t>
+          <t>2339I000795 - Biométrico  esta en sede cuenta como adicional no registra en el inventario de PCT</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1573</v>
-      </c>
-      <c r="B11" t="inlineStr"/>
+        <v>1548</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1548</v>
+      </c>
       <c r="C11" s="2" t="n">
         <v>46269</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>H_86189370e5df</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+          <t>H_981b2aa0739f</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MACANAL</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>SANTA ROSA DE VITERBO</t>
+          <t>MACANAL</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -23596,33 +23956,33 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>RECOLECCION</t>
+          <t>DENUNCIO</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2339I000795 - Biométrico  esta en sede cuenta como adicional no registra en el inventario de PCT</t>
+          <t>PAD DE FIRMAS: Se informa que el dispositivo se encuentra perdido. Debido a que el acta de asignación del elemento se encuentra debidamente firmada, se solicita realizar la respectiva denuncia por la pérdida del equipo y adelantar el procedimiento correspondiente.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1548</v>
+        <v>8601</v>
       </c>
       <c r="B12" t="n">
-        <v>1548</v>
+        <v>8601</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>H_981b2aa0739f</t>
+          <t>H_dfd3347a6a8e</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MACANAL</t>
+          <t>AGUAZUL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -23632,17 +23992,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>MACANAL</t>
+          <t>AGUAZUL</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Boyacá</t>
+          <t>Casanare</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -23652,38 +24012,38 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>DENUNCIO</t>
+          <t>RECOLECCION</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>PAD DE FIRMAS: Se informa que el dispositivo se encuentra perdido. Debido a que el acta de asignación del elemento se encuentra debidamente firmada, se solicita realizar la respectiva denuncia por la pérdida del equipo y adelantar el procedimiento correspondiente.</t>
+          <t>Biométrico está en sede cuenta como adicional</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>8601</v>
+        <v>7360</v>
       </c>
       <c r="B13" t="n">
-        <v>8601</v>
+        <v>1</v>
       </c>
       <c r="C13" s="2" t="n">
         <v>46273</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>H_dfd3347a6a8e</t>
+          <t>H_42bb652a9f00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>AGUAZUL</t>
+          <t>BODEGA COLSOF</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asignado</t>
+          <t>Pendiente Acta</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -23693,17 +24053,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>AGUAZUL</t>
+          <t>SARAVENA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Casanare</t>
+          <t>Arauca</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>GESTIONATECH</t>
+          <t>COBERTURA</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -23713,7 +24073,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Biométrico está en sede cuenta como adicional</t>
+          <t>Biométrico está en sede cuenta como adicional retirar de la sede</t>
         </is>
       </c>
     </row>
@@ -23729,7 +24089,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>H_42bb652a9f00</t>
+          <t>H_07553e1af367</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -23764,12 +24124,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>RECOLECCION</t>
+          <t>CAMBIO DE ESTADO A FACTURABLE</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Biométrico está en sede cuenta como adicional retirar de la sede</t>
+          <t>Biométrico está en uso actualmente, pero PCT se encuentra retirado</t>
         </is>
       </c>
     </row>
@@ -23778,29 +24138,29 @@
         <v>7360</v>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>7360</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>46273</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>H_07553e1af367</t>
+          <t>H_5aa503b8f03f</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BODEGA COLSOF</t>
+          <t>SARAVENA</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Pendiente Acta</t>
+          <t>Asignado</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -23820,33 +24180,33 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>CAMBIO DE ESTADO A FACTURABLE</t>
+          <t>DENUNCIO</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Biométrico está en uso actualmente, pero PCT se encuentra retirado</t>
+          <t>Biométrico está asignado, pero no está en la sede directora informa que se devolvió</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>7360</v>
+        <v>1395</v>
       </c>
       <c r="B16" t="n">
-        <v>7360</v>
+        <v>1395</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>H_5aa503b8f03f</t>
+          <t>H_a60c15475fb1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SARAVENA</t>
+          <t>URRAO</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -23856,114 +24216,100 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>SARAVENA</t>
+          <t>URRAO</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Arauca</t>
+          <t>Antioquia</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>COBERTURA</t>
+          <t>INSARED</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>DENUNCIO</t>
+          <t>RECOLECCION</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Biométrico está asignado, pero no está en la sede directora informa que se devolvió</t>
+          <t>La tablet serial 3109SH2020003393 actualmente, aparece asignada en PCT a la oficina 1395 – Antioquia – Urrao y en el inventario figura con la condición “NO facturable”. Sin embargo, durante la validación realizada, la directora de la oficina nos informa que la tablet fue trasladada a la oficina de Abejorral y que actualmente se encuentra en poder del señor Alejandro Ocampo Marín</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1399</v>
-      </c>
-      <c r="B17" t="n">
-        <v>1399</v>
-      </c>
+        <v>1577</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" s="2" t="n">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>H_2b1581fc161e</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>ZARAGOA</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Asignado</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
+          <t>H_28178afd14df</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ZARAGOZA</t>
+          <t>SOCOTA</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Antioquia</t>
+          <t>Boyacá</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>INSARED</t>
+          <t>GESTIONATECH</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>RECOLECCION</t>
+          <t>CAMBIO DE ESTADO A FACTURABLE</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Se encuentra el lector pin pad 1920233064 en la oficina de 1399 - ZARAGOZA en PCT aparece GARANTÍA FABRICANTE - INTERNO como retirado</t>
+          <t>Biométrico Adicional el director lo tiene en uso, no regsitra en PCT</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1395</v>
+        <v>1518</v>
       </c>
       <c r="B18" t="n">
-        <v>1395</v>
+        <v>1</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>H_a60c15475fb1</t>
+          <t>H_f3feb7409f8b</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>URRAO</t>
+          <t>BODEGA COLSOF</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asignado</t>
+          <t>Pendiente Acta</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -23973,17 +24319,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>URRAO</t>
+          <t>CHITA</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Antioquia</t>
+          <t>Boyacá</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>INSARED</t>
+          <t>GESTIONATECH</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -23993,34 +24339,48 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>La tablet serial 3109SH2020003393 actualmente, aparece asignada en PCT a la oficina 1395 – Antioquia – Urrao y en el inventario figura con la condición “NO facturable”. Sin embargo, durante la validación realizada, la directora de la oficina nos informa que la tablet fue trasladada a la oficina de Abejorral y que actualmente se encuentra en poder del señor Alejandro Ocampo Marín</t>
+          <t>Biométrico adicional recoger en la sede, esta en la oficina de CHITA pero tiene acta de retiro de GUEPSA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1577</v>
-      </c>
-      <c r="B19" t="inlineStr"/>
+        <v>3118</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3118</v>
+      </c>
       <c r="C19" s="2" t="n">
         <v>46275</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>H_28178afd14df</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>H_45cdd7b36374</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CHOCONTA</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>SOCOTA</t>
+          <t>CHOCONTA</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Boyacá</t>
+          <t>Cundinamarca</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -24030,53 +24390,53 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>CAMBIO DE ESTADO A FACTURABLE</t>
+          <t>DENUNCIO</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Biométrico Adicional el director lo tiene en uno, no regsitra en PCT</t>
+          <t>Se envia correo para realizar la denincia</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1518</v>
+        <v>6670</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>6670</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>46275</v>
+        <v>46274</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>H_f3feb7409f8b</t>
+          <t>H_64afd177463e</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BODEGA COLSOF</t>
+          <t>VENADILLO</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Pendiente Acta</t>
+          <t>Asignado</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CHITA</t>
+          <t>VENADILLO</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Boyacá</t>
+          <t>Tolima</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -24086,33 +24446,33 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>RECOLECCION</t>
+          <t>DENUNCIO</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Biométrico adicional recoger en la sede, esta en la oficina de CHITA pero tiene acta de retiro de GUEPSA</t>
+          <t>Biometrico no esta en la sede, se le envia correo al director para la denuncia</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3118</v>
+        <v>7910</v>
       </c>
       <c r="B21" t="n">
-        <v>3118</v>
+        <v>7910</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>H_45cdd7b36374</t>
+          <t>H_5a241b4d9918</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CHOCONTA</t>
+          <t>LA HORMIGA</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -24127,48 +24487,48 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CHOCONTA</t>
+          <t>LA HORMIGA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Cundinamarca</t>
+          <t>Putumayo</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>GESTIONATECH</t>
+          <t>COBERTURA</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>DENUNCIO</t>
+          <t>OPERACION</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Se envia correo para realizar la denincia</t>
+          <t>LA HORMIGA reportan falla de Lector de pin pad  1920077556. Director montó CATI para cambio.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>6670</v>
+        <v>1301</v>
       </c>
       <c r="B22" t="n">
-        <v>6670</v>
+        <v>1325</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>H_64afd177463e</t>
+          <t>H_52d6cf3f7e85</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>VENADILLO</t>
+          <t>CHIGORODO</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -24178,53 +24538,53 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>VENADILLO</t>
+          <t>ANDES</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Tolima</t>
+          <t>Antioquia</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>GESTIONATECH</t>
+          <t>INSARED</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>DENUNCIO</t>
+          <t>CAMBIO DE ESTADO A FACTURABLE</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Biometrico no esta en la sede, se le envia correo al director para la denuncia</t>
+          <t>TABLETA estan en el no facturable se encuentran en la oficina</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>7910</v>
+        <v>2405</v>
       </c>
       <c r="B23" t="n">
-        <v>7910</v>
+        <v>2405</v>
       </c>
       <c r="C23" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>H_5a241b4d9918</t>
+          <t>H_739528e71ff9</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LA HORMIGA</t>
+          <t>BECERRIL</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -24239,53 +24599,53 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>LA HORMIGA</t>
+          <t>BECERRIL</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Putumayo</t>
+          <t>Cesar</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>COBERTURA</t>
+          <t>GESTIONATECH</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>OPERACION</t>
+          <t>DENUNCIO</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>LA HORMIGA reportan falla de Lector de pin pad  1920077556. Director montó CATI para cambio.</t>
+          <t>Impresora perdida 49717265 PEREZ DIAZ PAOLA YANETH JESUS paolay.perez@bancoagrario.gov.co</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1301</v>
+        <v>1534</v>
       </c>
       <c r="B24" t="n">
-        <v>1325</v>
+        <v>1</v>
       </c>
       <c r="C24" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>H_52d6cf3f7e85</t>
+          <t>H_2661657889d7</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CHIGORODO</t>
+          <t>BODEGA COLSOF</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Asignado</t>
+          <t>Pendiente Acta</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -24295,17 +24655,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ANDES</t>
+          <t>GARAGOA</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Antioquia</t>
+          <t>Boyacá</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>INSARED</t>
+          <t>GESTIONATECH</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -24315,28 +24675,28 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>TABLETA estan en el no facturable se encuentran en la oficina</t>
+          <t>Se evidenció que el biométrico con serial 2432I014452 cuenta con un acta de retiro asociada al CATI IM3234330; sin embargo, actualmente el equipo se encuentra físicamente en la oficina y está siendo utilizado por la directora.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2405</v>
+        <v>1534</v>
       </c>
       <c r="B25" t="n">
-        <v>2405</v>
+        <v>1534</v>
       </c>
       <c r="C25" s="2" t="n">
         <v>46276</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>H_739528e71ff9</t>
+          <t>H_646fdca913af</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BECERRIL</t>
+          <t>GARAGOA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -24351,12 +24711,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>BECERRIL</t>
+          <t>GARAGOA</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Cesar</t>
+          <t>Boyacá</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -24371,23 +24731,23 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Impresora perdida 49717265 PEREZ DIAZ PAOLA YANETH JESUS paolay.perez@bancoagrario.gov.co</t>
+          <t>La directora informa que el biométrico con serial 2338018447, el cual figura asignado a la oficina en PCTriage, no se encuentra físicamente en las instalaciones y manifiesta que este equipo fue devuelto en relación con el caso anteriormente mencionado.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1534</v>
+        <v>1530</v>
       </c>
       <c r="B26" t="n">
         <v>1</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>H_2661657889d7</t>
+          <t>H_72befdb78ea8</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -24402,12 +24762,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>GARAGOA</t>
+          <t>CHIQUINQUIRA</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -24422,33 +24782,33 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>CAMBIO DE ESTADO A FACTURABLE</t>
+          <t>RECOLECCION</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Se evidenció que el biométrico con serial 2432I014452 cuenta con un acta de retiro asociada al CATI IM3234330; sin embargo, actualmente el equipo se encuentra físicamente en la oficina y está siendo utilizado por la directora.</t>
+          <t>1920232446 - ELEMENTO SOBRANTE EN LA OFICINA RECOLECTAR-Lector de banda pin pad</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1534</v>
+        <v>2701</v>
       </c>
       <c r="B27" t="n">
-        <v>1534</v>
+        <v>2701</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>H_646fdca913af</t>
+          <t>H_8bf8410babb9</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>GARAGOA</t>
+          <t>AYAPEL</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -24458,17 +24818,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>GARAGOA</t>
+          <t>AYAPEL</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Boyacá</t>
+          <t>Córdoba</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -24483,48 +24843,48 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>La directora informa que el biométrico con serial 2338018447, el cual figura asignado a la oficina en PCTriage, no se encuentra físicamente en las instalaciones y manifiesta que este equipo fue devuelto en relación con el caso anteriormente mencionado.</t>
+          <t>PAD de firmas  NO HACEN DENUNCIA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1530</v>
+        <v>8635</v>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>8635</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>H_72befdb78ea8</t>
+          <t>H_797f3092011a</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BODEGA COLSOF</t>
+          <t>PARATEBUENO</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Pendiente Acta</t>
+          <t>Asignado</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>CHIQUINQUIRA</t>
+          <t>PARATEBUENO</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Boyacá</t>
+          <t>Cundinamarca</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -24534,53 +24894,53 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>RECOLECCION</t>
+          <t>DENUNCIO</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>1920232446 - ELEMENTO SOBRANTE EN LA OFICINA RECOLECTAR-Lector de banda pin pad</t>
+          <t xml:space="preserve"> ELEMENTO PERDIDO- CASO Nº SD7195996" 86064291 - TORRES BENACHI FREDY </t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2701</v>
+        <v>6350</v>
       </c>
       <c r="B29" t="n">
-        <v>2701</v>
+        <v>1</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>H_8bf8410babb9</t>
+          <t>H_8342527939d4</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>AYAPEL</t>
+          <t>BODEGA COLSOF</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Asignado</t>
+          <t>Distribución</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>AYAPEL</t>
+          <t>OVEJAS</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Córdoba</t>
+          <t>Sucre</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -24590,53 +24950,39 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>DENUNCIO</t>
+          <t>RECOLECCION</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>PAD de firmas  NO HACEN DENUNCIA</t>
+          <t>Elemento sobrante LECTOR BIOMETRICO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>8635</v>
-      </c>
-      <c r="B30" t="n">
-        <v>8635</v>
-      </c>
+        <v>6350</v>
+      </c>
+      <c r="B30" t="inlineStr"/>
       <c r="C30" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>H_797f3092011a</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>PARATEBUENO</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Asignado</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
+          <t>H_6b0c9c60ff5a</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>PARATEBUENO</t>
+          <t>OVEJAS</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Cundinamarca</t>
+          <t>Sucre</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -24646,12 +24992,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>DENUNCIO</t>
+          <t>INETUM</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ELEMENTO PERDIDO- CASO Nº SD7195996" 86064291 - TORRES BENACHI FREDY </t>
+          <t>Biometrico pertenece al anterior proveedor</t>
         </is>
       </c>
     </row>
@@ -24660,29 +25006,29 @@
         <v>6350</v>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>6350</v>
       </c>
       <c r="C31" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>H_8342527939d4</t>
+          <t>H_06371ec95c39</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>BODEGA COLSOF</t>
+          <t>OVEJAS</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Distribución</t>
+          <t>Asignado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -24702,12 +25048,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>RECOLECCION</t>
+          <t>DENUNCIO</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Elemento sobrante LECTOR BIOMETRICO</t>
+          <t>Elementos perdidos  Lector biométrico 2338017569</t>
         </is>
       </c>
     </row>
@@ -24715,18 +25061,32 @@
       <c r="A32" t="n">
         <v>6350</v>
       </c>
-      <c r="B32" t="inlineStr"/>
+      <c r="B32" t="n">
+        <v>6350</v>
+      </c>
       <c r="C32" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>H_6b0c9c60ff5a</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+          <t>H_79964f56a3c0</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>OVEJAS</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>OVEJAS</t>
@@ -24742,25 +25102,47 @@
           <t>GESTIONATECH</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Pad de firmas 3HZQ001567 elemento perdido</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
         <v>6350</v>
       </c>
-      <c r="B33" t="inlineStr"/>
+      <c r="B33" t="n">
+        <v>6350</v>
+      </c>
       <c r="C33" s="2" t="n">
         <v>46280</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>H_896cf4ce30dd</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+          <t>H_bd87a5006614</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>OVEJAS</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>OVEJAS</t>
@@ -24776,8 +25158,16 @@
           <t>GESTIONATECH</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Biométrico 2432I012659  elemento perdido</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -24826,7 +25216,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>NOVEDAD</t>
+          <t>OPERACION</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -24836,270 +25226,954 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
+      <c r="A35" t="n">
+        <v>6639</v>
+      </c>
+      <c r="B35" t="n">
+        <v>6639</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>H_0c0f8ee7c221</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>HERRERA CORREGIMIENTO (DEL MUNICIPIO DE RIOBLANCO - TOLIMA)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>HERRERA Corregimiento (Del Municipio de Rioblanco - Tolima)</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Elementos registrados en inventario, pero que no se encuentran físicamente en la oficina-Pad de firmas: 3HZQ001731</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
+      <c r="A36" t="n">
+        <v>6639</v>
+      </c>
+      <c r="B36" t="n">
+        <v>6639</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>H_30fbb1046639</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>HERRERA CORREGIMIENTO (DEL MUNICIPIO DE RIOBLANCO - TOLIMA)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>HERRERA Corregimiento (Del Municipio de Rioblanco - Tolima)</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Elementos registrados en inventario, pero que no se encuentran físicamente en la oficina-Lector biométrico: 2432I014964</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
+      <c r="A37" t="n">
+        <v>6639</v>
+      </c>
+      <c r="B37" t="n">
+        <v>6639</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>H_2c0e33bbf017</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>HERRERA CORREGIMIENTO (DEL MUNICIPIO DE RIOBLANCO - TOLIMA)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>HERRERA Corregimiento (Del Municipio de Rioblanco - Tolima)</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Elementos registrados en inventario, pero que no se encuentran físicamente en la oficina-Lector biométrico: 2432I014985</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
+      <c r="A38" t="n">
+        <v>6639</v>
+      </c>
       <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
+      <c r="C38" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>H_4c98f60236e9</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>HERRERA Corregimiento (Del Municipio de Rioblanco - Tolima)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Elementos que se encuentran físicamente en la oficina, pero no aparecen registrados en el inventario: Pad de firmas: 3HZQ001727</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
+      <c r="A39" t="n">
+        <v>6639</v>
+      </c>
       <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
+      <c r="C39" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>H_400d5c725075</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>HERRERA Corregimiento (Del Municipio de Rioblanco - Tolima)</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Elementos que se encuentran físicamente en la oficina, pero no aparecen registrados en el inventario: Lector biométrico: 2432I014917</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
+      <c r="A40" t="n">
+        <v>6639</v>
+      </c>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
+      <c r="C40" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>H_b3d2a52d38f7</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>HERRERA Corregimiento (Del Municipio de Rioblanco - Tolima)</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Elementos que se encuentran físicamente en la oficina, pero no aparecen registrados en el inventario: Lector biométrico: 2432I014978</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
+      <c r="A41" t="n">
+        <v>6368</v>
+      </c>
+      <c r="B41" t="n">
+        <v>6368</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>H_8e4fc2753e76</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>SAN PEDRO</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>SAN PEDRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Sucre</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Elemento perdido Lector biométrico 2432I012842 - CASO MALETIN ROJO SD7197845- 64479056 - FLOREZ ARRIETA VERONICA SOFIA</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
+      <c r="A42" t="n">
+        <v>6646</v>
+      </c>
+      <c r="B42" t="n">
+        <v>6646</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>H_b603da0a6b43</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>RIOBLANCO</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>RIOBLANCO</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ASEGURAMIENTO</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>No se realiza acta de mantenimiento, ya que el director no firma porque la tableta se encuentra en la oficina de neiva y esta siendo utilizada, la tiene el coordinador control de inversion Faiver Artuduanga</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+      <c r="A43" t="n">
+        <v>7930</v>
+      </c>
+      <c r="B43" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>H_6d1a9c6e87db</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PUERTO ASIS</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>PUERTO ASIS</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Putumayo</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>COBERTURA</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>se realizó comunicación con el coordinador Faiver Artunduaga</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
+      <c r="A44" t="n">
+        <v>3913</v>
+      </c>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
+      <c r="C44" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>H_ea8857f5cbeb</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>GARZON</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Huila</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>CAMBIO DE ESTADO A FACTURABLE</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>TABLETA SE ENCUENTRA EN "NO" FACTURABLE SE ENCUENTRA SIENDO UTILIZADA EN LA OFICINA</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
+      <c r="A45" t="n">
+        <v>1501</v>
+      </c>
       <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
+      <c r="C45" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>H_5b19d4dbb15e</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>AQUITANIA</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Boyacá</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>ELEMENTOS PERDIDO, SE COLOCA DENUNCIA</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="A46" t="n">
+        <v>1379</v>
+      </c>
+      <c r="B46" t="n">
+        <v>1379</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>H_02368d2cf0d2</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>GUARNE</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>GUARNE</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>INSARED</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ASEGURAMIENTO</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Tablet correspondiente a la oficina de Guarne, registrada como NO facturable. Actualmente, el equipo se encuentra físicamente en la oficina de San Roqu</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
+      <c r="A47" t="n">
+        <v>1379</v>
+      </c>
       <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
+      <c r="C47" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>H_6b7a555a29e6</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>GUARNE</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>INSARED</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ASEGURAMIENTO</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Tablet que, de acuerdo con la información suministrada por el coordinador Jaime, corresponde al equipo que tiene asignado para la oficina de Guarne. Sin embargo, al realizar la validación en PC Triage, se evidencia que la tablet se encuentra asignada a la oficina de Antioquia – Titiribí</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="A48" t="n">
+        <v>1207</v>
+      </c>
+      <c r="B48" t="n">
+        <v>1207</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>H_916c7c600dfd</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>CARTAGENA</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>CARTAGENA</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>ELEMENTOS PERDIDOS, SE COLOCA DENUNCIA</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="A49" t="n">
+        <v>1207</v>
+      </c>
+      <c r="B49" t="n">
+        <v>1207</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>H_40768d0f5fdc</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>CARTAGENA</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>CARTAGENA</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>ELEMENTOS PERDIDOS, SE COLOCA DENUNCIA</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="A50" t="n">
+        <v>1207</v>
+      </c>
+      <c r="B50" t="n">
+        <v>1207</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>H_44935dd723de</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>CARTAGENA</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>CARTAGENA</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>ELEMENTOS PERDIDOS, SE COLOCA DENUNCIA</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
+      <c r="A51" t="n">
+        <v>2442</v>
+      </c>
       <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
+      <c r="C51" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>H_0fdd90ff6023</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>LA JAGUA DE IBIRICO</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Cesar</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>PERDIDO NUMERO DE CASOL SD7200893</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
+      <c r="A52" t="n">
+        <v>7950</v>
+      </c>
       <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
+      <c r="C52" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>H_41acdc50568a</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>VILLAGARZON</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Putumayo</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>COBERTURA</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>CAMBIO DE ESTADO A FACTURABLE</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>no esta en la oficina y tiene acta de retiro  Este fue el que llegó en reemplazo 2338018714.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
+      <c r="A53" t="n">
+        <v>1568</v>
+      </c>
       <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
+      <c r="C53" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>H_5233187062aa</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>SAMACA</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Boyacá</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>PIN PAD CUENTA CON ACTA DE RETIRO, PARA RECOLECCION</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>

</xml_diff>

<commit_message>
Ingesta diaria 2026-09-23 15:21
</commit_message>
<xml_diff>
--- a/data/Campos_actual.xlsx
+++ b/data/Campos_actual.xlsx
@@ -1190,7 +1190,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
@@ -5158,7 +5158,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -5494,7 +5494,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F205" t="inlineStr"/>
@@ -6226,7 +6226,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F207" t="inlineStr"/>
@@ -6342,7 +6342,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F214" t="inlineStr"/>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F215" t="inlineStr"/>
@@ -6652,7 +6652,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F312" t="inlineStr"/>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F319" t="inlineStr"/>
@@ -9880,7 +9880,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F334" t="inlineStr"/>
@@ -10036,7 +10036,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F340" t="inlineStr"/>
@@ -10312,7 +10312,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
@@ -10640,7 +10640,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F367" t="inlineStr"/>
@@ -11042,7 +11042,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F377" t="inlineStr"/>
@@ -11068,7 +11068,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F378" t="inlineStr"/>
@@ -11392,7 +11392,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F390" t="inlineStr"/>
@@ -11920,7 +11920,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F410" t="inlineStr"/>
@@ -12032,7 +12032,7 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F414" t="inlineStr"/>
@@ -12526,7 +12526,7 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>Reprogramada_Finalizada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F433" t="inlineStr"/>
@@ -12812,7 +12812,7 @@
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F444" t="inlineStr"/>
@@ -13684,7 +13684,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F476" t="inlineStr"/>
@@ -13710,7 +13710,7 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F477" t="inlineStr"/>
@@ -14690,7 +14690,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F511" t="inlineStr">
@@ -14798,7 +14798,7 @@
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F515" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F533" t="inlineStr"/>
@@ -15826,7 +15826,7 @@
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F553" t="inlineStr"/>
@@ -16454,7 +16454,7 @@
       </c>
       <c r="E577" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F577" t="inlineStr"/>
@@ -18242,7 +18242,7 @@
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F643" t="inlineStr"/>
@@ -18418,7 +18418,7 @@
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F649" t="inlineStr"/>
@@ -18698,7 +18698,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F659" t="inlineStr">
@@ -19128,7 +19128,7 @@
       </c>
       <c r="E674" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F674" t="inlineStr"/>
@@ -19180,7 +19180,7 @@
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F676" t="inlineStr"/>
@@ -19586,7 +19586,7 @@
       </c>
       <c r="E691" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F691" t="inlineStr"/>
@@ -19664,7 +19664,7 @@
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F694" t="inlineStr"/>
@@ -21732,7 +21732,7 @@
       </c>
       <c r="E766" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F766" t="inlineStr"/>
@@ -21826,7 +21826,7 @@
       </c>
       <c r="E769" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F769" t="inlineStr">
@@ -22516,7 +22516,7 @@
       </c>
       <c r="E794" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F794" t="inlineStr"/>
@@ -23248,7 +23248,7 @@
       </c>
       <c r="E822" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F822" t="inlineStr">
@@ -23280,7 +23280,7 @@
       </c>
       <c r="E823" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F823" t="inlineStr"/>
@@ -26176,23 +26176,49 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
+      <c r="A54" t="n">
+        <v>7370</v>
+      </c>
       <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
+      <c r="C54" s="2" t="n">
+        <v>46287</v>
+      </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TAME</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Arauca</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>COBERTURA</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>CAMBIO DE ESTADO A FACTURABLE</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Aparece ese PAD 1920232949 en la oficina. Y el 1920232090, q está en nuestro inventario no está en la oficina. @Santiago Noel Colsof se comunicó con el director  y deja correo para el respectivo denuncio.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" s="2" t="n">
+        <v>46287</v>
+      </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>

</xml_diff>

<commit_message>
Ingesta diaria 2026-09-25 10:26
</commit_message>
<xml_diff>
--- a/data/Campos_actual.xlsx
+++ b/data/Campos_actual.xlsx
@@ -696,7 +696,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
@@ -820,7 +824,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H12" t="n">
         <v>1</v>
       </c>
@@ -944,7 +952,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H16" t="n">
         <v>1</v>
       </c>
@@ -1003,8 +1015,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H18" t="n">
         <v>1</v>
       </c>
@@ -1029,8 +1049,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H19" t="n">
         <v>1</v>
       </c>
@@ -1060,7 +1088,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H20" t="n">
         <v>1</v>
       </c>
@@ -1085,8 +1117,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H21" t="n">
         <v>1</v>
       </c>
@@ -1111,8 +1151,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Con Cumplimiento de Fecha Inicio y Fin (Adelanto)</t>
+        </is>
+      </c>
       <c r="H22" t="n">
         <v>1</v>
       </c>
@@ -1142,7 +1190,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H23" t="n">
         <v>1</v>
       </c>
@@ -1167,8 +1219,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H24" t="n">
         <v>1</v>
       </c>
@@ -1467,8 +1527,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H34" t="n">
         <v>1</v>
       </c>
@@ -1579,8 +1647,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Con Cumplimiento de Fecha Inicio y Fin (Adelanto)</t>
+        </is>
+      </c>
       <c r="H38" t="n">
         <v>1</v>
       </c>
@@ -1657,8 +1733,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H41" t="n">
         <v>1</v>
       </c>
@@ -1735,8 +1819,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H44" t="n">
         <v>1</v>
       </c>
@@ -1784,7 +1876,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1938,7 +2030,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2110,7 +2202,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H57" t="n">
         <v>1</v>
       </c>
@@ -2187,8 +2283,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H60" t="n">
         <v>1</v>
       </c>
@@ -2299,8 +2403,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H64" t="n">
         <v>1</v>
       </c>
@@ -2330,7 +2442,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H65" t="n">
         <v>1</v>
       </c>
@@ -2355,8 +2471,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H66" t="n">
         <v>1</v>
       </c>
@@ -2433,8 +2557,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H69" t="n">
         <v>1</v>
       </c>
@@ -2605,8 +2737,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H75" t="n">
         <v>1</v>
       </c>
@@ -3300,7 +3440,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H100" t="n">
         <v>1</v>
       </c>
@@ -3356,7 +3500,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H102" t="n">
         <v>1</v>
       </c>
@@ -3537,8 +3685,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H109" t="n">
         <v>1</v>
       </c>
@@ -3612,7 +3768,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -3794,7 +3950,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -3898,7 +4054,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -4031,8 +4187,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H128" t="n">
         <v>1</v>
       </c>
@@ -4184,7 +4348,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -4236,7 +4400,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F136" t="inlineStr"/>
@@ -4418,7 +4582,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
@@ -4582,7 +4746,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H149" t="n">
         <v>1</v>
       </c>
@@ -4706,7 +4874,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H153" t="n">
         <v>1</v>
       </c>
@@ -4770,7 +4942,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H155" t="n">
         <v>1</v>
       </c>
@@ -4792,11 +4968,19 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H156" t="n">
         <v>1</v>
       </c>
@@ -4873,8 +5057,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H159" t="n">
         <v>1</v>
       </c>
@@ -4930,7 +5122,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr"/>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H161" t="n">
         <v>1</v>
       </c>
@@ -4978,7 +5174,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -5020,7 +5216,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H164" t="n">
         <v>1</v>
       </c>
@@ -5045,8 +5245,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H165" t="n">
         <v>1</v>
       </c>
@@ -5076,7 +5284,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H166" t="n">
         <v>1</v>
       </c>
@@ -5106,7 +5318,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H167" t="n">
         <v>1</v>
       </c>
@@ -5136,7 +5352,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr"/>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H168" t="n">
         <v>1</v>
       </c>
@@ -5364,7 +5584,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr"/>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H176" t="n">
         <v>1</v>
       </c>
@@ -5420,7 +5644,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H178" t="n">
         <v>1</v>
       </c>
@@ -5494,7 +5722,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -5658,7 +5886,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F187" t="inlineStr"/>
@@ -5833,8 +6061,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
-      <c r="G193" t="inlineStr"/>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H193" t="n">
         <v>1</v>
       </c>
@@ -5916,7 +6152,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G196" t="inlineStr"/>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H196" t="n">
         <v>1</v>
       </c>
@@ -5941,8 +6181,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F197" t="inlineStr"/>
-      <c r="G197" t="inlineStr"/>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H197" t="n">
         <v>1</v>
       </c>
@@ -6024,7 +6272,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H200" t="n">
         <v>1</v>
       </c>
@@ -6054,7 +6306,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H201" t="n">
         <v>1</v>
       </c>
@@ -6170,11 +6426,19 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>En proceso</t>
-        </is>
-      </c>
-      <c r="F205" t="inlineStr"/>
-      <c r="G205" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H205" t="n">
         <v>1</v>
       </c>
@@ -6204,7 +6468,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr"/>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H206" t="n">
         <v>1</v>
       </c>
@@ -6320,7 +6588,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G210" t="inlineStr"/>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H210" t="n">
         <v>1</v>
       </c>
@@ -6342,7 +6614,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -6379,8 +6651,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr"/>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H212" t="n">
         <v>1</v>
       </c>
@@ -6436,11 +6716,19 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>En proceso</t>
-        </is>
-      </c>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H214" t="n">
         <v>1</v>
       </c>
@@ -6488,7 +6776,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
@@ -6754,7 +7042,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -7044,7 +7332,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G234" t="inlineStr"/>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H234" t="n">
         <v>1</v>
       </c>
@@ -7134,7 +7426,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -7304,7 +7596,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -7372,7 +7664,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G244" t="inlineStr"/>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H244" t="n">
         <v>1</v>
       </c>
@@ -7470,7 +7766,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr"/>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H247" t="n">
         <v>1</v>
       </c>
@@ -7534,7 +7834,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr"/>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H249" t="n">
         <v>1</v>
       </c>
@@ -7590,7 +7894,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -7666,7 +7970,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr"/>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H253" t="n">
         <v>1</v>
       </c>
@@ -7832,7 +8140,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G258" t="inlineStr"/>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H258" t="n">
         <v>1</v>
       </c>
@@ -7862,7 +8174,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G259" t="inlineStr"/>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H259" t="n">
         <v>1</v>
       </c>
@@ -8038,7 +8354,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr"/>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H265" t="n">
         <v>1</v>
       </c>
@@ -8089,8 +8409,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr"/>
-      <c r="G267" t="inlineStr"/>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H267" t="n">
         <v>1</v>
       </c>
@@ -8193,8 +8521,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr"/>
-      <c r="G271" t="inlineStr"/>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H271" t="n">
         <v>1</v>
       </c>
@@ -8279,8 +8615,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr"/>
-      <c r="G274" t="inlineStr"/>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H274" t="n">
         <v>1</v>
       </c>
@@ -8425,8 +8769,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F279" t="inlineStr"/>
-      <c r="G279" t="inlineStr"/>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Con Cumplimiento de Fecha Inicio y Fin (Adelanto)</t>
+        </is>
+      </c>
       <c r="H279" t="n">
         <v>1</v>
       </c>
@@ -8503,8 +8855,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr"/>
-      <c r="G282" t="inlineStr"/>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H282" t="n">
         <v>1</v>
       </c>
@@ -8690,7 +9050,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G289" t="inlineStr"/>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H289" t="n">
         <v>1</v>
       </c>
@@ -8798,7 +9162,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G293" t="inlineStr"/>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H293" t="n">
         <v>1</v>
       </c>
@@ -8820,7 +9188,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F294" t="inlineStr"/>
@@ -9270,7 +9638,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G311" t="inlineStr"/>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H311" t="n">
         <v>1</v>
       </c>
@@ -9326,7 +9698,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G313" t="inlineStr"/>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H313" t="n">
         <v>1</v>
       </c>
@@ -9400,7 +9776,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F316" t="inlineStr"/>
@@ -9478,7 +9854,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F319" t="inlineStr"/>
@@ -9590,7 +9966,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G323" t="inlineStr"/>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Fin</t>
+        </is>
+      </c>
       <c r="H323" t="n">
         <v>1</v>
       </c>
@@ -9612,7 +9992,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -9620,7 +10000,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G324" t="inlineStr"/>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H324" t="n">
         <v>1</v>
       </c>
@@ -9650,7 +10034,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G325" t="inlineStr"/>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H325" t="n">
         <v>1</v>
       </c>
@@ -9727,8 +10115,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F328" t="inlineStr"/>
-      <c r="G328" t="inlineStr"/>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H328" t="n">
         <v>1</v>
       </c>
@@ -9805,8 +10201,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F331" t="inlineStr"/>
-      <c r="G331" t="inlineStr"/>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H331" t="n">
         <v>1</v>
       </c>
@@ -9854,11 +10258,19 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F333" t="inlineStr"/>
-      <c r="G333" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H333" t="n">
         <v>1</v>
       </c>
@@ -10406,7 +10818,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G353" t="inlineStr"/>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H353" t="n">
         <v>1</v>
       </c>
@@ -10436,7 +10852,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G354" t="inlineStr"/>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H354" t="n">
         <v>1</v>
       </c>
@@ -10565,8 +10985,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F359" t="inlineStr"/>
-      <c r="G359" t="inlineStr"/>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H359" t="n">
         <v>1</v>
       </c>
@@ -10614,7 +11042,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F361" t="inlineStr"/>
@@ -10640,7 +11068,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
@@ -10908,7 +11336,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F372" t="inlineStr"/>
@@ -10968,7 +11396,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G374" t="inlineStr"/>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H374" t="n">
         <v>1</v>
       </c>
@@ -11123,11 +11555,7 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F380" t="inlineStr">
-        <is>
-          <t>Finalizado</t>
-        </is>
-      </c>
+      <c r="F380" t="inlineStr"/>
       <c r="G380" t="inlineStr"/>
       <c r="H380" t="n">
         <v>1</v>
@@ -11332,7 +11760,7 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F388" t="inlineStr"/>
@@ -11392,7 +11820,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F390" t="inlineStr"/>
@@ -11920,7 +12348,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F410" t="inlineStr"/>
@@ -12058,7 +12486,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F415" t="inlineStr"/>
@@ -12191,8 +12619,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F420" t="inlineStr"/>
-      <c r="G420" t="inlineStr"/>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H420" t="n">
         <v>1</v>
       </c>
@@ -13010,7 +13446,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G451" t="inlineStr"/>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H451" t="n">
         <v>1</v>
       </c>
@@ -13040,7 +13480,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G452" t="inlineStr"/>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H452" t="n">
         <v>1</v>
       </c>
@@ -13070,7 +13514,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G453" t="inlineStr"/>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H453" t="n">
         <v>1</v>
       </c>
@@ -13134,7 +13582,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G455" t="inlineStr"/>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Fin</t>
+        </is>
+      </c>
       <c r="H455" t="n">
         <v>1</v>
       </c>
@@ -13159,8 +13611,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F456" t="inlineStr"/>
-      <c r="G456" t="inlineStr"/>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H456" t="n">
         <v>1</v>
       </c>
@@ -13190,7 +13650,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G457" t="inlineStr"/>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H457" t="n">
         <v>1</v>
       </c>
@@ -13215,8 +13679,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F458" t="inlineStr"/>
-      <c r="G458" t="inlineStr"/>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H458" t="n">
         <v>1</v>
       </c>
@@ -13272,7 +13744,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G460" t="inlineStr"/>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H460" t="n">
         <v>1</v>
       </c>
@@ -13297,8 +13773,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F461" t="inlineStr"/>
-      <c r="G461" t="inlineStr"/>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H461" t="n">
         <v>1</v>
       </c>
@@ -13323,8 +13807,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F462" t="inlineStr"/>
-      <c r="G462" t="inlineStr"/>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H462" t="n">
         <v>1</v>
       </c>
@@ -14004,7 +14496,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G488" t="inlineStr"/>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H488" t="n">
         <v>1</v>
       </c>
@@ -14136,7 +14632,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G492" t="inlineStr"/>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H492" t="n">
         <v>2</v>
       </c>
@@ -14161,8 +14661,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F493" t="inlineStr"/>
-      <c r="G493" t="inlineStr"/>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H493" t="n">
         <v>1</v>
       </c>
@@ -14362,7 +14870,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G499" t="inlineStr"/>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H499" t="n">
         <v>1</v>
       </c>
@@ -14462,7 +14974,7 @@
       </c>
       <c r="E503" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F503" t="inlineStr"/>
@@ -14496,7 +15008,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G504" t="inlineStr"/>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H504" t="n">
         <v>1</v>
       </c>
@@ -14667,8 +15183,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F510" t="inlineStr"/>
-      <c r="G510" t="inlineStr"/>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H510" t="n">
         <v>1</v>
       </c>
@@ -14690,7 +15214,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F511" t="inlineStr">
@@ -14698,7 +15222,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G511" t="inlineStr"/>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H511" t="n">
         <v>1</v>
       </c>
@@ -14806,7 +15334,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G515" t="inlineStr"/>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H515" t="n">
         <v>1</v>
       </c>
@@ -15070,7 +15602,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G525" t="inlineStr"/>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H525" t="n">
         <v>1</v>
       </c>
@@ -15254,7 +15790,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G531" t="inlineStr"/>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H531" t="n">
         <v>1</v>
       </c>
@@ -15302,7 +15842,7 @@
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F533" t="inlineStr"/>
@@ -15336,7 +15876,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G534" t="inlineStr"/>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H534" t="n">
         <v>1</v>
       </c>
@@ -15361,8 +15905,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F535" t="inlineStr"/>
-      <c r="G535" t="inlineStr"/>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H535" t="n">
         <v>1</v>
       </c>
@@ -15436,7 +15988,7 @@
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F538" t="inlineStr"/>
@@ -15621,8 +16173,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F545" t="inlineStr"/>
-      <c r="G545" t="inlineStr"/>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H545" t="n">
         <v>1</v>
       </c>
@@ -16068,7 +16628,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G562" t="inlineStr"/>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H562" t="n">
         <v>1</v>
       </c>
@@ -16558,7 +17122,7 @@
       </c>
       <c r="E581" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F581" t="inlineStr"/>
@@ -17267,8 +17831,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F606" t="inlineStr"/>
-      <c r="G606" t="inlineStr"/>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G606" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H606" t="n">
         <v>1</v>
       </c>
@@ -17319,8 +17891,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F608" t="inlineStr"/>
-      <c r="G608" t="inlineStr"/>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G608" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H608" t="n">
         <v>1</v>
       </c>
@@ -18245,8 +18825,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F643" t="inlineStr"/>
-      <c r="G643" t="inlineStr"/>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H643" t="n">
         <v>1</v>
       </c>
@@ -18294,7 +18882,7 @@
       </c>
       <c r="E645" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F645" t="inlineStr">
@@ -18418,11 +19006,19 @@
       </c>
       <c r="E649" t="inlineStr">
         <is>
-          <t>En proceso</t>
-        </is>
-      </c>
-      <c r="F649" t="inlineStr"/>
-      <c r="G649" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H649" t="n">
         <v>1</v>
       </c>
@@ -18530,7 +19126,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G653" t="inlineStr"/>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H653" t="n">
         <v>1</v>
       </c>
@@ -18555,8 +19155,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F654" t="inlineStr"/>
-      <c r="G654" t="inlineStr"/>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H654" t="n">
         <v>1</v>
       </c>
@@ -18646,7 +19254,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G657" t="inlineStr"/>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H657" t="n">
         <v>1</v>
       </c>
@@ -18676,7 +19288,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G658" t="inlineStr"/>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H658" t="n">
         <v>1</v>
       </c>
@@ -18706,7 +19322,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G659" t="inlineStr"/>
+      <c r="G659" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H659" t="n">
         <v>1</v>
       </c>
@@ -18796,7 +19416,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G662" t="inlineStr"/>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H662" t="n">
         <v>1</v>
       </c>
@@ -18860,7 +19484,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G664" t="inlineStr"/>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H664" t="n">
         <v>1</v>
       </c>
@@ -18916,7 +19544,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G666" t="inlineStr"/>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H666" t="n">
         <v>1</v>
       </c>
@@ -18972,7 +19604,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G668" t="inlineStr"/>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H668" t="n">
         <v>1</v>
       </c>
@@ -19028,7 +19664,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G670" t="inlineStr"/>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H670" t="n">
         <v>1</v>
       </c>
@@ -19105,8 +19745,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F673" t="inlineStr"/>
-      <c r="G673" t="inlineStr"/>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H673" t="n">
         <v>1</v>
       </c>
@@ -19157,8 +19805,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F675" t="inlineStr"/>
-      <c r="G675" t="inlineStr"/>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H675" t="n">
         <v>1</v>
       </c>
@@ -19180,7 +19836,7 @@
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F676" t="inlineStr"/>
@@ -19214,7 +19870,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G677" t="inlineStr"/>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H677" t="n">
         <v>1</v>
       </c>
@@ -19270,7 +19930,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G679" t="inlineStr"/>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H679" t="n">
         <v>1</v>
       </c>
@@ -19300,7 +19964,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G680" t="inlineStr"/>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H680" t="n">
         <v>1</v>
       </c>
@@ -19460,7 +20128,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G686" t="inlineStr"/>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H686" t="n">
         <v>1</v>
       </c>
@@ -19511,8 +20183,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F688" t="inlineStr"/>
-      <c r="G688" t="inlineStr"/>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H688" t="n">
         <v>1</v>
       </c>
@@ -19664,7 +20344,7 @@
       </c>
       <c r="E694" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F694" t="inlineStr"/>
@@ -19690,7 +20370,7 @@
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F695" t="inlineStr"/>
@@ -19750,7 +20430,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G697" t="inlineStr"/>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H697" t="n">
         <v>1</v>
       </c>
@@ -19910,7 +20594,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G703" t="inlineStr"/>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H703" t="n">
         <v>1</v>
       </c>
@@ -20029,8 +20717,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F707" t="inlineStr"/>
-      <c r="G707" t="inlineStr"/>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H707" t="n">
         <v>1</v>
       </c>
@@ -20060,7 +20756,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G708" t="inlineStr"/>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H708" t="n">
         <v>1</v>
       </c>
@@ -20158,7 +20858,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G711" t="inlineStr"/>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H711" t="n">
         <v>1</v>
       </c>
@@ -20266,7 +20970,7 @@
       </c>
       <c r="E715" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F715" t="inlineStr">
@@ -20394,7 +21098,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G719" t="inlineStr"/>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H719" t="n">
         <v>1</v>
       </c>
@@ -20536,7 +21244,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G724" t="inlineStr"/>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H724" t="n">
         <v>1</v>
       </c>
@@ -20566,7 +21278,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G725" t="inlineStr"/>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H725" t="n">
         <v>1</v>
       </c>
@@ -20617,8 +21333,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F727" t="inlineStr"/>
-      <c r="G727" t="inlineStr"/>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H727" t="n">
         <v>1</v>
       </c>
@@ -20643,8 +21367,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F728" t="inlineStr"/>
-      <c r="G728" t="inlineStr"/>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H728" t="n">
         <v>1</v>
       </c>
@@ -20794,7 +21526,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G733" t="inlineStr"/>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H733" t="n">
         <v>1</v>
       </c>
@@ -20957,8 +21693,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F739" t="inlineStr"/>
-      <c r="G739" t="inlineStr"/>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H739" t="n">
         <v>1</v>
       </c>
@@ -21309,8 +22053,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F751" t="inlineStr"/>
-      <c r="G751" t="inlineStr"/>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H751" t="n">
         <v>1</v>
       </c>
@@ -21335,8 +22087,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F752" t="inlineStr"/>
-      <c r="G752" t="inlineStr"/>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H752" t="n">
         <v>1</v>
       </c>
@@ -21361,8 +22121,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F753" t="inlineStr"/>
-      <c r="G753" t="inlineStr"/>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H753" t="n">
         <v>1</v>
       </c>
@@ -21392,7 +22160,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G754" t="inlineStr"/>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H754" t="n">
         <v>1</v>
       </c>
@@ -21422,7 +22194,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G755" t="inlineStr"/>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H755" t="n">
         <v>1</v>
       </c>
@@ -21452,7 +22228,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G756" t="inlineStr"/>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H756" t="n">
         <v>1</v>
       </c>
@@ -21482,7 +22262,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G757" t="inlineStr"/>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H757" t="n">
         <v>1</v>
       </c>
@@ -21538,7 +22322,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G759" t="inlineStr"/>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H759" t="n">
         <v>1</v>
       </c>
@@ -21568,7 +22356,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G760" t="inlineStr"/>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H760" t="n">
         <v>1</v>
       </c>
@@ -21598,7 +22390,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G761" t="inlineStr"/>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H761" t="n">
         <v>1</v>
       </c>
@@ -21623,8 +22419,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F762" t="inlineStr"/>
-      <c r="G762" t="inlineStr"/>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H762" t="n">
         <v>1</v>
       </c>
@@ -21931,8 +22735,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F772" t="inlineStr"/>
-      <c r="G772" t="inlineStr"/>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H772" t="n">
         <v>1</v>
       </c>
@@ -21991,8 +22803,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F774" t="inlineStr"/>
-      <c r="G774" t="inlineStr"/>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H774" t="n">
         <v>1</v>
       </c>
@@ -22516,7 +23336,7 @@
       </c>
       <c r="E794" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F794" t="inlineStr"/>
@@ -22630,8 +23450,10 @@
       </c>
     </row>
     <row r="799">
-      <c r="A799" t="n">
-        <v>3000</v>
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
       </c>
       <c r="B799" t="inlineStr">
         <is>
@@ -22656,8 +23478,10 @@
       </c>
     </row>
     <row r="800">
-      <c r="A800" t="n">
-        <v>1800</v>
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
       </c>
       <c r="B800" t="inlineStr">
         <is>
@@ -22682,8 +23506,10 @@
       </c>
     </row>
     <row r="801">
-      <c r="A801" t="n">
-        <v>1600</v>
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
       </c>
       <c r="B801" t="inlineStr">
         <is>
@@ -22708,8 +23534,10 @@
       </c>
     </row>
     <row r="802">
-      <c r="A802" t="n">
-        <v>6900</v>
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>6900</t>
+        </is>
       </c>
       <c r="B802" t="inlineStr">
         <is>
@@ -22742,8 +23570,10 @@
       </c>
     </row>
     <row r="803">
-      <c r="A803" t="n">
-        <v>1500</v>
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
       </c>
       <c r="B803" t="inlineStr">
         <is>
@@ -22794,8 +23624,10 @@
       </c>
     </row>
     <row r="805">
-      <c r="A805" t="n">
-        <v>3900</v>
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>3900</t>
+        </is>
       </c>
       <c r="B805" t="inlineStr">
         <is>
@@ -22844,8 +23676,10 @@
       <c r="H806" t="inlineStr"/>
     </row>
     <row r="807">
-      <c r="A807" t="n">
-        <v>1411</v>
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>1411</t>
+        </is>
       </c>
       <c r="B807" t="inlineStr">
         <is>
@@ -22916,12 +23750,14 @@
       <c r="H809" t="inlineStr"/>
     </row>
     <row r="810">
-      <c r="A810" t="n">
-        <v>1600</v>
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>01600-J</t>
+        </is>
       </c>
       <c r="B810" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Barranquilla</t>
+          <t>JEFATURA BARRANQUILLA</t>
         </is>
       </c>
       <c r="C810" s="2" t="n">
@@ -22940,12 +23776,14 @@
       <c r="H810" t="inlineStr"/>
     </row>
     <row r="811">
-      <c r="A811" t="n">
-        <v>3000</v>
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>03000-J</t>
+        </is>
       </c>
       <c r="B811" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Bogotá COB</t>
+          <t>JEFATURA BOGOTA</t>
         </is>
       </c>
       <c r="C811" s="2" t="n">
@@ -22964,12 +23802,14 @@
       <c r="H811" t="inlineStr"/>
     </row>
     <row r="812">
-      <c r="A812" t="n">
-        <v>3000</v>
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>03000-J</t>
+        </is>
       </c>
       <c r="B812" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Villavicencio</t>
+          <t>JEFATURA VILLAVICENCIO</t>
         </is>
       </c>
       <c r="C812" s="2" t="n">
@@ -22980,7 +23820,7 @@
       </c>
       <c r="E812" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F812" t="inlineStr"/>
@@ -22988,12 +23828,14 @@
       <c r="H812" t="inlineStr"/>
     </row>
     <row r="813">
-      <c r="A813" t="n">
-        <v>1300</v>
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>01300-J</t>
+        </is>
       </c>
       <c r="B813" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Medellin COB</t>
+          <t>JEFATURA MEDELLIN</t>
         </is>
       </c>
       <c r="C813" s="2" t="n">
@@ -23020,12 +23862,14 @@
       <c r="H813" t="inlineStr"/>
     </row>
     <row r="814">
-      <c r="A814" t="n">
-        <v>1300</v>
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>01300-J</t>
+        </is>
       </c>
       <c r="B814" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Monteria</t>
+          <t>JEFATURA MONTERIA</t>
         </is>
       </c>
       <c r="C814" s="2" t="n">
@@ -23044,12 +23888,14 @@
       <c r="H814" t="inlineStr"/>
     </row>
     <row r="815">
-      <c r="A815" t="n">
-        <v>6900</v>
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>06900-J</t>
+        </is>
       </c>
       <c r="B815" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Cali COB</t>
+          <t>JEFATURA CALI</t>
         </is>
       </c>
       <c r="C815" s="2" t="n">
@@ -23068,12 +23914,14 @@
       <c r="H815" t="inlineStr"/>
     </row>
     <row r="816">
-      <c r="A816" t="n">
-        <v>6900</v>
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>06900-J</t>
+        </is>
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Pasto</t>
+          <t>JEFATURA PASTO</t>
         </is>
       </c>
       <c r="C816" s="2" t="n">
@@ -23096,12 +23944,14 @@
       <c r="H816" t="inlineStr"/>
     </row>
     <row r="817">
-      <c r="A817" t="n">
-        <v>6900</v>
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>06900-J</t>
+        </is>
       </c>
       <c r="B817" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones POPAYAN</t>
+          <t>JEFATURA POPAYAN</t>
         </is>
       </c>
       <c r="C817" s="2" t="n">
@@ -23124,12 +23974,14 @@
       <c r="H817" t="inlineStr"/>
     </row>
     <row r="818">
-      <c r="A818" t="n">
-        <v>1600</v>
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>01600-J</t>
+        </is>
       </c>
       <c r="B818" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones SINCELEJO</t>
+          <t>JEFATUTA SINCELEJO</t>
         </is>
       </c>
       <c r="C818" s="2" t="n">
@@ -23152,12 +24004,14 @@
       <c r="H818" t="inlineStr"/>
     </row>
     <row r="819">
-      <c r="A819" t="n">
-        <v>1600</v>
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>01600-J</t>
+        </is>
       </c>
       <c r="B819" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Valledupar</t>
+          <t>JEFATURA VALLEDUPAR</t>
         </is>
       </c>
       <c r="C819" s="2" t="n">
@@ -23176,12 +24030,14 @@
       <c r="H819" t="inlineStr"/>
     </row>
     <row r="820">
-      <c r="A820" t="n">
-        <v>1800</v>
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>01800-J</t>
+        </is>
       </c>
       <c r="B820" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Manizales COB</t>
+          <t>JEFATURA MANIZALES</t>
         </is>
       </c>
       <c r="C820" s="2" t="n">
@@ -23200,12 +24056,14 @@
       <c r="H820" t="inlineStr"/>
     </row>
     <row r="821">
-      <c r="A821" t="n">
-        <v>1500</v>
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>01500-J</t>
+        </is>
       </c>
       <c r="B821" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Tunja COB</t>
+          <t>JEFATURA TUNJA</t>
         </is>
       </c>
       <c r="C821" s="2" t="n">
@@ -23232,12 +24090,14 @@
       <c r="H821" t="inlineStr"/>
     </row>
     <row r="822">
-      <c r="A822" t="n">
-        <v>6000</v>
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>06000-J</t>
+        </is>
       </c>
       <c r="B822" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Bucaramanga COB</t>
+          <t>JEFATURA BUCARAMANGA</t>
         </is>
       </c>
       <c r="C822" s="2" t="n">
@@ -23264,12 +24124,14 @@
       <c r="H822" t="inlineStr"/>
     </row>
     <row r="823">
-      <c r="A823" t="n">
-        <v>6000</v>
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>06000-J</t>
+        </is>
       </c>
       <c r="B823" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Cúcuta COB</t>
+          <t>JEFATURA CUCUTA</t>
         </is>
       </c>
       <c r="C823" s="2" t="n">
@@ -23288,12 +24150,14 @@
       <c r="H823" t="inlineStr"/>
     </row>
     <row r="824">
-      <c r="A824" t="n">
-        <v>3900</v>
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>03900-J</t>
+        </is>
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones Neiva COB</t>
+          <t>JEFATURA NEIVA</t>
         </is>
       </c>
       <c r="C824" s="2" t="n">
@@ -23312,12 +24176,14 @@
       <c r="H824" t="inlineStr"/>
     </row>
     <row r="825">
-      <c r="A825" t="n">
-        <v>3900</v>
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>03900-J</t>
+        </is>
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>Jefatura de Operaciones IBAGUE</t>
+          <t>JEFATURA IBAGUE</t>
         </is>
       </c>
       <c r="C825" s="2" t="n">
@@ -26214,34 +27080,88 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
+      <c r="A55" t="n">
+        <v>5117</v>
+      </c>
       <c r="B55" t="inlineStr"/>
       <c r="C55" s="2" t="n">
-        <v>46287</v>
-      </c>
-      <c r="D55" t="inlineStr"/>
+        <v>46289</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>H_0d964dea0f5b</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>CUCUTILLA</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>PIN PAD: 1920040811 - sobrante para recoleccion</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
+      <c r="A56" t="n">
+        <v>3144</v>
+      </c>
       <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
+      <c r="C56" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>H_1e3e1e781cae</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>LA PEÑA</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Cundinamarca</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Lector biométrico  2338016493 - sobrante para recoleccion</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>

</xml_diff>

<commit_message>
Ingesta diaria 2026-09-28 11:54
</commit_message>
<xml_diff>
--- a/data/Campos_actual.xlsx
+++ b/data/Campos_actual.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -4080,7 +4080,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -4968,7 +4968,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -7962,7 +7962,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -8312,7 +8312,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -9880,7 +9880,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F320" t="inlineStr"/>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
@@ -10112,7 +10112,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
@@ -10198,7 +10198,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
@@ -10344,7 +10344,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F342" t="inlineStr"/>
@@ -10534,7 +10534,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
@@ -10620,7 +10620,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F346" t="inlineStr"/>
@@ -11180,7 +11180,7 @@
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F366" t="inlineStr"/>
@@ -11258,7 +11258,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F369" t="inlineStr"/>
@@ -11734,7 +11734,7 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F387" t="inlineStr"/>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>Finalizada</t>
+          <t>Reprogramada_Finalizada</t>
         </is>
       </c>
       <c r="F433" t="inlineStr"/>
@@ -14384,7 +14384,7 @@
       </c>
       <c r="E484" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F484" t="inlineStr"/>
@@ -15816,7 +15816,7 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F532" t="inlineStr"/>
@@ -15988,7 +15988,7 @@
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F538" t="inlineStr"/>
@@ -17724,7 +17724,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F602" t="inlineStr"/>
@@ -17750,7 +17750,7 @@
       </c>
       <c r="E603" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F603" t="inlineStr"/>
@@ -17802,7 +17802,7 @@
       </c>
       <c r="E605" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F605" t="inlineStr"/>
@@ -17862,7 +17862,7 @@
       </c>
       <c r="E607" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F607" t="inlineStr"/>
@@ -19212,7 +19212,7 @@
       </c>
       <c r="E656" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F656" t="inlineStr">
@@ -19246,7 +19246,7 @@
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F657" t="inlineStr">
@@ -20370,7 +20370,7 @@
       </c>
       <c r="E695" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F695" t="inlineStr"/>
@@ -20944,7 +20944,7 @@
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F714" t="inlineStr"/>
@@ -21998,7 +21998,7 @@
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F749" t="inlineStr"/>
@@ -22886,7 +22886,7 @@
       </c>
       <c r="E777" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F777" t="inlineStr">
@@ -23414,7 +23414,7 @@
       </c>
       <c r="E797" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F797" t="inlineStr"/>
@@ -23880,7 +23880,7 @@
       </c>
       <c r="E814" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F814" t="inlineStr"/>
@@ -27164,60 +27164,214 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
+      <c r="A57" t="n">
+        <v>6649</v>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>H_1a176920409d</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>BODEGA COLSOF</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Pendiente Acta</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>ATACO</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Elementos que se encuentran físicamente en la oficina, pero no aparecen registrados en el inventari</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
+      <c r="A58" t="n">
+        <v>6649</v>
+      </c>
       <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
+      <c r="C58" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>H_3c6e5085736f</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>ATACO</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Elementos registrados en inventario, pero que no se encuentran físicamente en la oficina</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
+      <c r="A59" t="n">
+        <v>6649</v>
+      </c>
+      <c r="B59" t="n">
+        <v>6649</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>H_b636329764c8</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ATACO</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>ATACO</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>CATI: SD7209959 TABLETA LA TIENE EL COORDINADOR DE CONTROL DE INVERSION faiver.artunduaga@bancoagrario.gov.co la va devolver a la sede de ibague</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
+      <c r="A60" t="n">
+        <v>6649</v>
+      </c>
+      <c r="B60" t="n">
+        <v>6649</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>H_4733c6dd14a7</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ATACO</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Asignado</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>ATACO</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>TABLETA ESTA EN LA OFICINA RECOLECCION</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>

</xml_diff>

<commit_message>
Ingesta diaria 2026-09-30 14:57
</commit_message>
<xml_diff>
--- a/data/Campos_actual.xlsx
+++ b/data/Campos_actual.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2097,8 +2097,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H40" t="n">
         <v>1</v>
       </c>
@@ -2494,7 +2502,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2914,7 +2922,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3165,8 +3173,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H67" t="n">
         <v>1</v>
       </c>
@@ -3521,8 +3537,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H76" t="n">
         <v>1</v>
       </c>
@@ -3750,7 +3774,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -3825,8 +3849,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H84" t="n">
         <v>1</v>
       </c>
@@ -3933,8 +3965,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H87" t="n">
         <v>1</v>
       </c>
@@ -4502,7 +4542,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4809,8 +4849,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H110" t="n">
         <v>1</v>
       </c>
@@ -4914,7 +4962,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5061,8 +5109,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H117" t="n">
         <v>1</v>
       </c>
@@ -5166,7 +5222,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5238,7 +5294,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5822,7 +5878,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -5933,8 +5989,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr"/>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H141" t="n">
         <v>1</v>
       </c>
@@ -6110,7 +6174,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
@@ -6185,8 +6249,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H148" t="n">
         <v>1</v>
       </c>
@@ -6598,7 +6670,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F158" t="inlineStr"/>
@@ -7061,8 +7133,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H169" t="n">
         <v>1</v>
       </c>
@@ -7641,8 +7721,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H184" t="n">
         <v>1</v>
       </c>
@@ -7945,8 +8033,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr"/>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H192" t="n">
         <v>1</v>
       </c>
@@ -8025,8 +8121,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F194" t="inlineStr"/>
-      <c r="G194" t="inlineStr"/>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H194" t="n">
         <v>1</v>
       </c>
@@ -8221,8 +8325,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr"/>
-      <c r="G199" t="inlineStr"/>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H199" t="n">
         <v>1</v>
       </c>
@@ -8557,8 +8669,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F207" t="inlineStr"/>
-      <c r="G207" t="inlineStr"/>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H207" t="n">
         <v>1</v>
       </c>
@@ -9698,7 +9818,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -9918,7 +10038,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -10909,8 +11029,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F263" t="inlineStr"/>
-      <c r="G263" t="inlineStr"/>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H263" t="n">
         <v>1</v>
       </c>
@@ -11033,8 +11161,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F266" t="inlineStr"/>
-      <c r="G266" t="inlineStr"/>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H266" t="n">
         <v>1</v>
       </c>
@@ -11066,7 +11202,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -11149,8 +11285,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F269" t="inlineStr"/>
-      <c r="G269" t="inlineStr"/>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H269" t="n">
         <v>1</v>
       </c>
@@ -11182,11 +11326,19 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F270" t="inlineStr"/>
-      <c r="G270" t="inlineStr"/>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H270" t="n">
         <v>1</v>
       </c>
@@ -11342,7 +11494,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -11709,8 +11861,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
-      <c r="G283" t="inlineStr"/>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H283" t="n">
         <v>1</v>
       </c>
@@ -11745,8 +11905,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr"/>
-      <c r="G284" t="inlineStr"/>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H284" t="n">
         <v>1</v>
       </c>
@@ -11781,8 +11949,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr"/>
-      <c r="G285" t="inlineStr"/>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H285" t="n">
         <v>1</v>
       </c>
@@ -11817,8 +11993,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr"/>
-      <c r="G286" t="inlineStr"/>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H286" t="n">
         <v>1</v>
       </c>
@@ -12041,8 +12225,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F292" t="inlineStr"/>
-      <c r="G292" t="inlineStr"/>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H292" t="n">
         <v>1</v>
       </c>
@@ -12265,8 +12457,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F298" t="inlineStr"/>
-      <c r="G298" t="inlineStr"/>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H298" t="n">
         <v>1</v>
       </c>
@@ -13694,7 +13894,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F336" t="inlineStr"/>
@@ -13918,7 +14118,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F342" t="inlineStr"/>
@@ -13954,7 +14154,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
@@ -14070,7 +14270,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F346" t="inlineStr"/>
@@ -14418,7 +14618,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F355" t="inlineStr"/>
@@ -14562,7 +14762,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
@@ -15010,7 +15210,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F371" t="inlineStr"/>
@@ -15162,7 +15362,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F375" t="inlineStr"/>
@@ -15273,8 +15473,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F378" t="inlineStr"/>
-      <c r="G378" t="inlineStr"/>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H378" t="n">
         <v>1</v>
       </c>
@@ -15306,7 +15514,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F379" t="inlineStr"/>
@@ -15414,7 +15622,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F382" t="inlineStr"/>
@@ -15450,7 +15658,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F383" t="inlineStr"/>
@@ -15937,8 +16145,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F396" t="inlineStr"/>
-      <c r="G396" t="inlineStr"/>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H396" t="n">
         <v>1</v>
       </c>
@@ -15973,8 +16189,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F397" t="inlineStr"/>
-      <c r="G397" t="inlineStr"/>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H397" t="n">
         <v>1</v>
       </c>
@@ -16330,7 +16554,7 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F407" t="inlineStr"/>
@@ -16366,7 +16590,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F408" t="inlineStr"/>
@@ -17282,7 +17506,7 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>Reprogramada_Finalizada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F433" t="inlineStr"/>
@@ -17354,7 +17578,7 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F435" t="inlineStr"/>
@@ -17390,7 +17614,7 @@
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F436" t="inlineStr"/>
@@ -18857,8 +19081,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F474" t="inlineStr"/>
-      <c r="G474" t="inlineStr"/>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H474" t="n">
         <v>1</v>
       </c>
@@ -19214,7 +19446,7 @@
       </c>
       <c r="E484" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F484" t="inlineStr"/>
@@ -19250,7 +19482,7 @@
       </c>
       <c r="E485" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F485" t="inlineStr"/>
@@ -19534,7 +19766,7 @@
       </c>
       <c r="E492" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F492" t="inlineStr">
@@ -19578,7 +19810,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F493" t="inlineStr">
@@ -20549,8 +20781,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F517" t="inlineStr"/>
-      <c r="G517" t="inlineStr"/>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H517" t="n">
         <v>1</v>
       </c>
@@ -21126,11 +21366,19 @@
       </c>
       <c r="E532" t="inlineStr">
         <is>
-          <t>En proceso</t>
-        </is>
-      </c>
-      <c r="F532" t="inlineStr"/>
-      <c r="G532" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H532" t="n">
         <v>1</v>
       </c>
@@ -21289,8 +21537,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F536" t="inlineStr"/>
-      <c r="G536" t="inlineStr"/>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H536" t="n">
         <v>1</v>
       </c>
@@ -21469,8 +21725,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F541" t="inlineStr"/>
-      <c r="G541" t="inlineStr"/>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H541" t="n">
         <v>1</v>
       </c>
@@ -23074,7 +23338,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F585" t="inlineStr">
@@ -23154,7 +23418,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F587" t="inlineStr">
@@ -23242,7 +23506,7 @@
       </c>
       <c r="E589" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F589" t="inlineStr">
@@ -23322,7 +23586,7 @@
       </c>
       <c r="E591" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F591" t="inlineStr">
@@ -23449,8 +23713,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F594" t="inlineStr"/>
-      <c r="G594" t="inlineStr"/>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H594" t="n">
         <v>1</v>
       </c>
@@ -23485,8 +23757,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F595" t="inlineStr"/>
-      <c r="G595" t="inlineStr"/>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H595" t="n">
         <v>1</v>
       </c>
@@ -23593,8 +23873,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F598" t="inlineStr"/>
-      <c r="G598" t="inlineStr"/>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H598" t="n">
         <v>1</v>
       </c>
@@ -23734,7 +24022,7 @@
       </c>
       <c r="E602" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F602" t="inlineStr"/>
@@ -23806,7 +24094,7 @@
       </c>
       <c r="E604" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F604" t="inlineStr"/>
@@ -23922,7 +24210,7 @@
       </c>
       <c r="E607" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F607" t="inlineStr"/>
@@ -24326,7 +24614,7 @@
       </c>
       <c r="E618" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F618" t="inlineStr"/>
@@ -24581,8 +24869,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F625" t="inlineStr"/>
-      <c r="G625" t="inlineStr"/>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H625" t="n">
         <v>1</v>
       </c>
@@ -24730,7 +25026,7 @@
       </c>
       <c r="E629" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F629" t="inlineStr"/>
@@ -24802,7 +25098,7 @@
       </c>
       <c r="E631" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F631" t="inlineStr"/>
@@ -25057,8 +25353,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F638" t="inlineStr"/>
-      <c r="G638" t="inlineStr"/>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H638" t="n">
         <v>1</v>
       </c>
@@ -25209,8 +25513,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F642" t="inlineStr"/>
-      <c r="G642" t="inlineStr"/>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H642" t="n">
         <v>1</v>
       </c>
@@ -25289,8 +25601,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F644" t="inlineStr"/>
-      <c r="G644" t="inlineStr"/>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H644" t="n">
         <v>1</v>
       </c>
@@ -25410,7 +25730,11 @@
           <t>Finalizado</t>
         </is>
       </c>
-      <c r="G647" t="inlineStr"/>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Fin (Adelanto)</t>
+        </is>
+      </c>
       <c r="H647" t="n">
         <v>1</v>
       </c>
@@ -25442,7 +25766,7 @@
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F648" t="inlineStr">
@@ -25566,7 +25890,7 @@
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F651" t="inlineStr"/>
@@ -26153,8 +26477,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F665" t="inlineStr"/>
-      <c r="G665" t="inlineStr"/>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H665" t="n">
         <v>1</v>
       </c>
@@ -26793,8 +27125,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F681" t="inlineStr"/>
-      <c r="G681" t="inlineStr"/>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H681" t="n">
         <v>1</v>
       </c>
@@ -26829,8 +27169,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F682" t="inlineStr"/>
-      <c r="G682" t="inlineStr"/>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H682" t="n">
         <v>1</v>
       </c>
@@ -26901,8 +27249,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F684" t="inlineStr"/>
-      <c r="G684" t="inlineStr"/>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H684" t="n">
         <v>1</v>
       </c>
@@ -27346,7 +27702,7 @@
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F696" t="inlineStr"/>
@@ -27426,7 +27782,7 @@
       </c>
       <c r="E698" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F698" t="inlineStr"/>
@@ -27501,8 +27857,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F700" t="inlineStr"/>
-      <c r="G700" t="inlineStr"/>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H700" t="n">
         <v>1</v>
       </c>
@@ -28041,8 +28405,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F713" t="inlineStr"/>
-      <c r="G713" t="inlineStr"/>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H713" t="n">
         <v>1</v>
       </c>
@@ -28074,7 +28446,7 @@
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F714" t="inlineStr"/>
@@ -29001,7 +29373,11 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F737" t="inlineStr"/>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
       <c r="G737" t="inlineStr"/>
       <c r="H737" t="n">
         <v>1</v>
@@ -29478,7 +29854,7 @@
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F749" t="inlineStr"/>
@@ -31050,7 +31426,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F788" t="inlineStr"/>
@@ -31842,7 +32218,7 @@
     <row r="810">
       <c r="A810" t="inlineStr">
         <is>
-          <t>01600-J</t>
+          <t>01600-BQUILLA</t>
         </is>
       </c>
       <c r="B810" t="inlineStr">
@@ -31878,7 +32254,7 @@
     <row r="811">
       <c r="A811" t="inlineStr">
         <is>
-          <t>03000-J</t>
+          <t>03000-BOGOTA</t>
         </is>
       </c>
       <c r="B811" t="inlineStr">
@@ -31914,7 +32290,7 @@
     <row r="812">
       <c r="A812" t="inlineStr">
         <is>
-          <t>03000-J</t>
+          <t>03000-VILLAO</t>
         </is>
       </c>
       <c r="B812" t="inlineStr">
@@ -31950,7 +32326,7 @@
     <row r="813">
       <c r="A813" t="inlineStr">
         <is>
-          <t>01300-J</t>
+          <t>01300-MEDELLIN</t>
         </is>
       </c>
       <c r="B813" t="inlineStr">
@@ -31994,7 +32370,7 @@
     <row r="814">
       <c r="A814" t="inlineStr">
         <is>
-          <t>01300-J</t>
+          <t>01300-J-MONTERIA</t>
         </is>
       </c>
       <c r="B814" t="inlineStr">
@@ -32030,7 +32406,7 @@
     <row r="815">
       <c r="A815" t="inlineStr">
         <is>
-          <t>06900-J</t>
+          <t>06900-CALI</t>
         </is>
       </c>
       <c r="B815" t="inlineStr">
@@ -32066,7 +32442,7 @@
     <row r="816">
       <c r="A816" t="inlineStr">
         <is>
-          <t>06900-J</t>
+          <t>06900-PASTO</t>
         </is>
       </c>
       <c r="B816" t="inlineStr">
@@ -32106,7 +32482,7 @@
     <row r="817">
       <c r="A817" t="inlineStr">
         <is>
-          <t>06900-J</t>
+          <t>06900-POPAYAN</t>
         </is>
       </c>
       <c r="B817" t="inlineStr">
@@ -32146,7 +32522,7 @@
     <row r="818">
       <c r="A818" t="inlineStr">
         <is>
-          <t>01600-J</t>
+          <t>01600-SINCELEJO</t>
         </is>
       </c>
       <c r="B818" t="inlineStr">
@@ -32186,7 +32562,7 @@
     <row r="819">
       <c r="A819" t="inlineStr">
         <is>
-          <t>01600-J</t>
+          <t>01600-VALLEDUPAR</t>
         </is>
       </c>
       <c r="B819" t="inlineStr">
@@ -32222,7 +32598,7 @@
     <row r="820">
       <c r="A820" t="inlineStr">
         <is>
-          <t>01800-J</t>
+          <t>01800-MANIZALES</t>
         </is>
       </c>
       <c r="B820" t="inlineStr">
@@ -32258,7 +32634,7 @@
     <row r="821">
       <c r="A821" t="inlineStr">
         <is>
-          <t>01500-J</t>
+          <t>01500-TUNJA</t>
         </is>
       </c>
       <c r="B821" t="inlineStr">
@@ -32302,7 +32678,7 @@
     <row r="822">
       <c r="A822" t="inlineStr">
         <is>
-          <t>06000-J</t>
+          <t>06000-BMANGA</t>
         </is>
       </c>
       <c r="B822" t="inlineStr">
@@ -32346,7 +32722,7 @@
     <row r="823">
       <c r="A823" t="inlineStr">
         <is>
-          <t>06000-J</t>
+          <t>06000-CUCUTA</t>
         </is>
       </c>
       <c r="B823" t="inlineStr">
@@ -32382,7 +32758,7 @@
     <row r="824">
       <c r="A824" t="inlineStr">
         <is>
-          <t>03900-J</t>
+          <t>03900-NEIVA</t>
         </is>
       </c>
       <c r="B824" t="inlineStr">
@@ -32418,7 +32794,7 @@
     <row r="825">
       <c r="A825" t="inlineStr">
         <is>
-          <t>03900-J</t>
+          <t>03900-IBAGUE</t>
         </is>
       </c>
       <c r="B825" t="inlineStr">
@@ -32470,7 +32846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L493"/>
+  <dimension ref="A1:L494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32562,7 +32938,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -32618,7 +32994,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -32674,7 +33050,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -32730,7 +33106,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -32786,7 +33162,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -32811,7 +33187,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Biométrico se encuentra como siniestro hurto pero en realidad esta en la oficina en uso operativo, se encuentra como "NO" facturable, Ssi no se aprueba se debe recoger</t>
+          <t>Biométrico se encuentra como siniestro hurto pero en realidad esta en la oficina en uso operativo, se encuentra como "NO" facturable, Si no se aprueba se debe recoger</t>
         </is>
       </c>
     </row>
@@ -32842,7 +33218,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -32898,7 +33274,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -32954,7 +33330,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -33052,7 +33428,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -33108,7 +33484,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -33164,7 +33540,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -33220,7 +33596,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -33276,7 +33652,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -33332,7 +33708,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -33365,18 +33741,32 @@
       <c r="A17" t="n">
         <v>1577</v>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
       <c r="C17" s="2" t="n">
         <v>46275</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>H_28178afd14df</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+          <t>H_4c475f212be3</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BODEGA COLSOF</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Pendiente Acta</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>SOCOTA</t>
@@ -33399,7 +33789,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Biométrico Adicional el director lo tiene en uso, no regsitra en PCT</t>
+          <t>Biométrico Adicional el director lo tiene en uso, STOCK COLSOF</t>
         </is>
       </c>
     </row>
@@ -33430,7 +33820,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -33486,7 +33876,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -33542,7 +33932,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -33598,7 +33988,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -33654,7 +34044,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -33710,7 +34100,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -33766,7 +34156,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -33822,7 +34212,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -33990,7 +34380,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -34046,7 +34436,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -34144,7 +34534,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -34200,7 +34590,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -34256,7 +34646,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -34312,7 +34702,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -34368,7 +34758,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -34424,7 +34814,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -34480,7 +34870,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -34662,7 +35052,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -34718,7 +35108,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -35012,7 +35402,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -35068,7 +35458,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -35124,7 +35514,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -35440,7 +35830,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -35538,7 +35928,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -35594,7 +35984,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -35624,46 +36014,138 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
+      <c r="A61" t="n">
+        <v>1510</v>
+      </c>
       <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
+      <c r="C61" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>H_6a05a729bc7d</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>CUBARA</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Boyacá</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>GESTIONATECH</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>DENUNCIO</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>BIOMETRICO SE ENCUENTRA PERDIDO, se envia correo para denuncia</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
+      <c r="A62" t="n">
+        <v>2128</v>
+      </c>
       <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
+      <c r="C62" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>H_46e34f0526be</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>BUENOS AIRES</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Cauca</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>INSARED</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ASEGURADORA</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> novedad con el equipo 5CD331DF46, SE ENCUENTRA ACTIVO Y ASIGNADO A LA OFICINA</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
+      <c r="A63" t="n">
+        <v>7310</v>
+      </c>
       <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
+      <c r="C63" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>H_c0e5395b3b13</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>CRAVO NORTE</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Arauca</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>COBERTURA</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>RECOLECCION</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Biométrico q no está en el inventario</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
@@ -41685,6 +42167,20 @@
       <c r="K493" t="inlineStr"/>
       <c r="L493" t="inlineStr"/>
     </row>
+    <row r="494">
+      <c r="A494" t="inlineStr"/>
+      <c r="B494" t="inlineStr"/>
+      <c r="C494" t="inlineStr"/>
+      <c r="D494" t="inlineStr"/>
+      <c r="E494" t="inlineStr"/>
+      <c r="F494" t="inlineStr"/>
+      <c r="G494" t="inlineStr"/>
+      <c r="H494" t="inlineStr"/>
+      <c r="I494" t="inlineStr"/>
+      <c r="J494" t="inlineStr"/>
+      <c r="K494" t="inlineStr"/>
+      <c r="L494" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ingesta diaria 2026-10-02 15:54
</commit_message>
<xml_diff>
--- a/data/Campos_actual.xlsx
+++ b/data/Campos_actual.xlsx
@@ -758,7 +758,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -805,8 +805,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H9" t="n">
         <v>1</v>
       </c>
@@ -1006,7 +1014,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1182,7 +1190,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2221,8 +2229,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H43" t="n">
         <v>1</v>
       </c>
@@ -2301,8 +2317,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H45" t="n">
         <v>1</v>
       </c>
@@ -2922,7 +2946,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3454,7 +3478,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3622,7 +3646,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -3813,8 +3837,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H83" t="n">
         <v>1</v>
       </c>
@@ -4089,8 +4121,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H90" t="n">
         <v>1</v>
       </c>
@@ -4246,7 +4286,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4321,8 +4361,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H96" t="n">
         <v>1</v>
       </c>
@@ -4429,8 +4477,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Con Cumplimiento de Fecha Inicio y Fin (Adelanto)</t>
+        </is>
+      </c>
       <c r="H99" t="n">
         <v>1</v>
       </c>
@@ -4509,8 +4565,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H101" t="n">
         <v>1</v>
       </c>
@@ -4625,8 +4689,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H104" t="n">
         <v>1</v>
       </c>
@@ -4893,8 +4965,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H111" t="n">
         <v>1</v>
       </c>
@@ -4929,8 +5009,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H112" t="n">
         <v>1</v>
       </c>
@@ -5294,7 +5382,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5333,8 +5421,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H123" t="n">
         <v>1</v>
       </c>
@@ -5629,8 +5725,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H131" t="n">
         <v>1</v>
       </c>
@@ -5809,8 +5913,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H136" t="n">
         <v>1</v>
       </c>
@@ -5842,7 +5954,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
@@ -6290,7 +6402,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -6381,8 +6493,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H151" t="n">
         <v>1</v>
       </c>
@@ -7177,8 +7297,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H170" t="n">
         <v>1</v>
       </c>
@@ -7533,8 +7661,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H179" t="n">
         <v>1</v>
       </c>
@@ -7569,8 +7705,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H180" t="n">
         <v>1</v>
       </c>
@@ -7765,8 +7909,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H185" t="n">
         <v>1</v>
       </c>
@@ -7873,8 +8025,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F188" t="inlineStr"/>
-      <c r="G188" t="inlineStr"/>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H188" t="n">
         <v>1</v>
       </c>
@@ -8289,8 +8449,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr"/>
-      <c r="G198" t="inlineStr"/>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H198" t="n">
         <v>1</v>
       </c>
@@ -9162,7 +9330,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F219" t="inlineStr"/>
@@ -10382,7 +10550,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -10470,7 +10638,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -10778,7 +10946,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -10913,8 +11081,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F260" t="inlineStr"/>
-      <c r="G260" t="inlineStr"/>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H260" t="n">
         <v>1</v>
       </c>
@@ -10993,8 +11169,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F262" t="inlineStr"/>
-      <c r="G262" t="inlineStr"/>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H262" t="n">
         <v>1</v>
       </c>
@@ -11494,7 +11678,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -11541,8 +11725,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr"/>
-      <c r="G275" t="inlineStr"/>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H275" t="n">
         <v>1</v>
       </c>
@@ -11621,8 +11813,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F277" t="inlineStr"/>
-      <c r="G277" t="inlineStr"/>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H277" t="n">
         <v>1</v>
       </c>
@@ -11814,7 +12014,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -12037,8 +12237,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr"/>
-      <c r="G287" t="inlineStr"/>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H287" t="n">
         <v>1</v>
       </c>
@@ -12150,11 +12358,19 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Programada</t>
-        </is>
-      </c>
-      <c r="F290" t="inlineStr"/>
-      <c r="G290" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H290" t="n">
         <v>1</v>
       </c>
@@ -12189,8 +12405,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr"/>
-      <c r="G291" t="inlineStr"/>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H291" t="n">
         <v>1</v>
       </c>
@@ -12385,8 +12609,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F296" t="inlineStr"/>
-      <c r="G296" t="inlineStr"/>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H296" t="n">
         <v>1</v>
       </c>
@@ -12421,8 +12653,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr"/>
-      <c r="G297" t="inlineStr"/>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H297" t="n">
         <v>1</v>
       </c>
@@ -13626,7 +13866,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F329" t="inlineStr"/>
@@ -13742,7 +13982,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F332" t="inlineStr"/>
@@ -13966,7 +14206,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F338" t="inlineStr"/>
@@ -14201,8 +14441,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F344" t="inlineStr"/>
-      <c r="G344" t="inlineStr"/>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H344" t="n">
         <v>1</v>
       </c>
@@ -14618,7 +14866,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F355" t="inlineStr"/>
@@ -15514,7 +15762,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F379" t="inlineStr"/>
@@ -15553,8 +15801,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F380" t="inlineStr"/>
-      <c r="G380" t="inlineStr"/>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H380" t="n">
         <v>1</v>
       </c>
@@ -16233,8 +16489,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F398" t="inlineStr"/>
-      <c r="G398" t="inlineStr"/>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H398" t="n">
         <v>1</v>
       </c>
@@ -16269,8 +16533,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F399" t="inlineStr"/>
-      <c r="G399" t="inlineStr"/>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H399" t="n">
         <v>1</v>
       </c>
@@ -16521,8 +16793,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F406" t="inlineStr"/>
-      <c r="G406" t="inlineStr"/>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H406" t="n">
         <v>1</v>
       </c>
@@ -16554,11 +16834,19 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>En proceso</t>
-        </is>
-      </c>
-      <c r="F407" t="inlineStr"/>
-      <c r="G407" t="inlineStr"/>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H407" t="n">
         <v>1</v>
       </c>
@@ -16593,8 +16881,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F408" t="inlineStr"/>
-      <c r="G408" t="inlineStr"/>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H408" t="n">
         <v>1</v>
       </c>
@@ -16745,8 +17041,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F412" t="inlineStr"/>
-      <c r="G412" t="inlineStr"/>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H412" t="n">
         <v>1</v>
       </c>
@@ -16781,8 +17085,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F413" t="inlineStr"/>
-      <c r="G413" t="inlineStr"/>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H413" t="n">
         <v>1</v>
       </c>
@@ -16817,8 +17129,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F414" t="inlineStr"/>
-      <c r="G414" t="inlineStr"/>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>Con Cumplimiento de Fecha Inicio y Fin (Adelanto)</t>
+        </is>
+      </c>
       <c r="H414" t="n">
         <v>1</v>
       </c>
@@ -16925,8 +17245,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr"/>
-      <c r="G417" t="inlineStr"/>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H417" t="n">
         <v>1</v>
       </c>
@@ -17185,8 +17513,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F424" t="inlineStr"/>
-      <c r="G424" t="inlineStr"/>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H424" t="n">
         <v>1</v>
       </c>
@@ -17650,7 +17986,7 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F437" t="inlineStr"/>
@@ -17938,7 +18274,7 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F445" t="inlineStr"/>
@@ -19482,7 +19818,7 @@
       </c>
       <c r="E485" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F485" t="inlineStr"/>
@@ -20121,8 +20457,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F500" t="inlineStr"/>
-      <c r="G500" t="inlineStr"/>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H500" t="n">
         <v>1</v>
       </c>
@@ -20229,8 +20573,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F503" t="inlineStr"/>
-      <c r="G503" t="inlineStr"/>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H503" t="n">
         <v>1</v>
       </c>
@@ -20502,7 +20854,7 @@
       </c>
       <c r="E510" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F510" t="inlineStr">
@@ -20629,8 +20981,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F513" t="inlineStr"/>
-      <c r="G513" t="inlineStr"/>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H513" t="n">
         <v>1</v>
       </c>
@@ -20969,8 +21329,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F522" t="inlineStr"/>
-      <c r="G522" t="inlineStr"/>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H522" t="n">
         <v>1</v>
       </c>
@@ -21002,7 +21370,7 @@
       </c>
       <c r="E523" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F523" t="inlineStr"/>
@@ -21157,8 +21525,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F527" t="inlineStr"/>
-      <c r="G527" t="inlineStr"/>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H527" t="n">
         <v>1</v>
       </c>
@@ -22173,8 +22549,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F553" t="inlineStr"/>
-      <c r="G553" t="inlineStr"/>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H553" t="n">
         <v>1</v>
       </c>
@@ -22350,7 +22734,7 @@
       </c>
       <c r="E558" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F558" t="inlineStr"/>
@@ -22386,7 +22770,7 @@
       </c>
       <c r="E559" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="F559" t="inlineStr"/>
@@ -23258,7 +23642,7 @@
       </c>
       <c r="E583" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F583" t="inlineStr"/>
@@ -23338,7 +23722,7 @@
       </c>
       <c r="E585" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F585" t="inlineStr">
@@ -23385,8 +23769,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F586" t="inlineStr"/>
-      <c r="G586" t="inlineStr"/>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H586" t="n">
         <v>1</v>
       </c>
@@ -23418,7 +23810,7 @@
       </c>
       <c r="E587" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F587" t="inlineStr">
@@ -23586,7 +23978,7 @@
       </c>
       <c r="E591" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F591" t="inlineStr">
@@ -23666,7 +24058,7 @@
       </c>
       <c r="E593" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F593" t="inlineStr">
@@ -23837,8 +24229,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F597" t="inlineStr"/>
-      <c r="G597" t="inlineStr"/>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H597" t="n">
         <v>1</v>
       </c>
@@ -23989,8 +24389,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F601" t="inlineStr"/>
-      <c r="G601" t="inlineStr"/>
+      <c r="F601" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H601" t="n">
         <v>1</v>
       </c>
@@ -24329,8 +24737,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F610" t="inlineStr"/>
-      <c r="G610" t="inlineStr"/>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G610" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H610" t="n">
         <v>1</v>
       </c>
@@ -24910,7 +25326,7 @@
       </c>
       <c r="E626" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F626" t="inlineStr">
@@ -25766,7 +26182,7 @@
       </c>
       <c r="E648" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F648" t="inlineStr">
@@ -26006,7 +26422,7 @@
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F654" t="inlineStr">
@@ -26053,8 +26469,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F655" t="inlineStr"/>
-      <c r="G655" t="inlineStr"/>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H655" t="n">
         <v>1</v>
       </c>
@@ -26309,8 +26733,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F661" t="inlineStr"/>
-      <c r="G661" t="inlineStr"/>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H661" t="n">
         <v>1</v>
       </c>
@@ -27001,8 +27433,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F678" t="inlineStr"/>
-      <c r="G678" t="inlineStr"/>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H678" t="n">
         <v>1</v>
       </c>
@@ -27702,7 +28142,7 @@
       </c>
       <c r="E696" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F696" t="inlineStr"/>
@@ -27821,8 +28261,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F699" t="inlineStr"/>
-      <c r="G699" t="inlineStr"/>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H699" t="n">
         <v>1</v>
       </c>
@@ -28017,8 +28465,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F704" t="inlineStr"/>
-      <c r="G704" t="inlineStr"/>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H704" t="n">
         <v>1</v>
       </c>
@@ -28138,7 +28594,7 @@
       </c>
       <c r="E707" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F707" t="inlineStr">
@@ -28449,8 +28905,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F714" t="inlineStr"/>
-      <c r="G714" t="inlineStr"/>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>Con Incumplimiento de Fecha Inicio y Fin</t>
+        </is>
+      </c>
       <c r="H714" t="n">
         <v>1</v>
       </c>
@@ -28686,7 +29150,7 @@
       </c>
       <c r="E720" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F720" t="inlineStr"/>
@@ -28929,8 +29393,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F726" t="inlineStr"/>
-      <c r="G726" t="inlineStr"/>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H726" t="n">
         <v>1</v>
       </c>
@@ -29337,8 +29809,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F736" t="inlineStr"/>
-      <c r="G736" t="inlineStr"/>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H736" t="n">
         <v>1</v>
       </c>
@@ -30237,8 +30717,16 @@
           <t>Programada</t>
         </is>
       </c>
-      <c r="F758" t="inlineStr"/>
-      <c r="G758" t="inlineStr"/>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H758" t="n">
         <v>1</v>
       </c>
@@ -31022,7 +31510,7 @@
       </c>
       <c r="E777" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F777" t="inlineStr">
@@ -31678,7 +32166,7 @@
       </c>
       <c r="E795" t="inlineStr">
         <is>
-          <t>Programada</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="F795" t="inlineStr"/>
@@ -32741,8 +33229,16 @@
           <t>Finalizada</t>
         </is>
       </c>
-      <c r="F823" t="inlineStr"/>
-      <c r="G823" t="inlineStr"/>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H823" t="inlineStr"/>
       <c r="I823" t="inlineStr">
         <is>
@@ -32777,8 +33273,16 @@
           <t>En proceso</t>
         </is>
       </c>
-      <c r="F824" t="inlineStr"/>
-      <c r="G824" t="inlineStr"/>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>Finalizado</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>OK - Cumplen Fechas Cronograma</t>
+        </is>
+      </c>
       <c r="H824" t="inlineStr"/>
       <c r="I824" t="inlineStr">
         <is>

</xml_diff>